<commit_message>
Updated filename and added new data.
</commit_message>
<xml_diff>
--- a/price_extractor.xlsx
+++ b/price_extractor.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AM23"/>
+  <dimension ref="A1:BE23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -624,6 +624,96 @@
           <t>Price_2025-02-25 21:06</t>
         </is>
       </c>
+      <c r="AN1" s="1" t="inlineStr">
+        <is>
+          <t>Product Name_2025-02-26 03:05</t>
+        </is>
+      </c>
+      <c r="AO1" s="1" t="inlineStr">
+        <is>
+          <t>Price_2025-02-26 03:05</t>
+        </is>
+      </c>
+      <c r="AP1" s="1" t="inlineStr">
+        <is>
+          <t>Product Name_2025-02-27 03:04</t>
+        </is>
+      </c>
+      <c r="AQ1" s="1" t="inlineStr">
+        <is>
+          <t>Price_2025-02-27 03:04</t>
+        </is>
+      </c>
+      <c r="AR1" s="1" t="inlineStr">
+        <is>
+          <t>Product Name_2025-02-28 03:05</t>
+        </is>
+      </c>
+      <c r="AS1" s="1" t="inlineStr">
+        <is>
+          <t>Price_2025-02-28 03:05</t>
+        </is>
+      </c>
+      <c r="AT1" s="1" t="inlineStr">
+        <is>
+          <t>Product Name_2025-03-01 03:04</t>
+        </is>
+      </c>
+      <c r="AU1" s="1" t="inlineStr">
+        <is>
+          <t>Price_2025-03-01 03:04</t>
+        </is>
+      </c>
+      <c r="AV1" s="1" t="inlineStr">
+        <is>
+          <t>Product Name_2025-03-02 03:05</t>
+        </is>
+      </c>
+      <c r="AW1" s="1" t="inlineStr">
+        <is>
+          <t>Price_2025-03-02 03:05</t>
+        </is>
+      </c>
+      <c r="AX1" s="1" t="inlineStr">
+        <is>
+          <t>Product Name_2025-03-03 03:05</t>
+        </is>
+      </c>
+      <c r="AY1" s="1" t="inlineStr">
+        <is>
+          <t>Price_2025-03-03 03:05</t>
+        </is>
+      </c>
+      <c r="AZ1" s="1" t="inlineStr">
+        <is>
+          <t>Product Name_2025-03-04 03:04</t>
+        </is>
+      </c>
+      <c r="BA1" s="1" t="inlineStr">
+        <is>
+          <t>Price_2025-03-04 03:04</t>
+        </is>
+      </c>
+      <c r="BB1" s="1" t="inlineStr">
+        <is>
+          <t>Product Name_2025-03-04 10:51</t>
+        </is>
+      </c>
+      <c r="BC1" s="1" t="inlineStr">
+        <is>
+          <t>Price_2025-03-04 10:51</t>
+        </is>
+      </c>
+      <c r="BD1" s="1" t="inlineStr">
+        <is>
+          <t>Product Name_2025-03-04 17:48</t>
+        </is>
+      </c>
+      <c r="BE1" s="1" t="inlineStr">
+        <is>
+          <t>Price_2025-03-04 17:48</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -821,6 +911,96 @@
           <t>2.679</t>
         </is>
       </c>
+      <c r="AN2" t="inlineStr">
+        <is>
+          <t>UNLEADED 87 (10% ETH)</t>
+        </is>
+      </c>
+      <c r="AO2" t="inlineStr">
+        <is>
+          <t>2.679</t>
+        </is>
+      </c>
+      <c r="AP2" t="inlineStr">
+        <is>
+          <t>UNLEADED 87 (10% ETH)</t>
+        </is>
+      </c>
+      <c r="AQ2" t="inlineStr">
+        <is>
+          <t>2.629</t>
+        </is>
+      </c>
+      <c r="AR2" t="inlineStr">
+        <is>
+          <t>UNLEADED 87 (10% ETH)</t>
+        </is>
+      </c>
+      <c r="AS2" t="inlineStr">
+        <is>
+          <t>2.629</t>
+        </is>
+      </c>
+      <c r="AT2" t="inlineStr">
+        <is>
+          <t>UNLEADED 87 (10% ETH)</t>
+        </is>
+      </c>
+      <c r="AU2" t="inlineStr">
+        <is>
+          <t>2.599</t>
+        </is>
+      </c>
+      <c r="AV2" t="inlineStr">
+        <is>
+          <t>UNLEADED 87 (10% ETH)</t>
+        </is>
+      </c>
+      <c r="AW2" t="inlineStr">
+        <is>
+          <t>2.599</t>
+        </is>
+      </c>
+      <c r="AX2" t="inlineStr">
+        <is>
+          <t>UNLEADED 87 (10% ETH)</t>
+        </is>
+      </c>
+      <c r="AY2" t="inlineStr">
+        <is>
+          <t>2.599</t>
+        </is>
+      </c>
+      <c r="AZ2" t="inlineStr">
+        <is>
+          <t>UNLEADED 87 (10% ETH)</t>
+        </is>
+      </c>
+      <c r="BA2" t="inlineStr">
+        <is>
+          <t>2.899</t>
+        </is>
+      </c>
+      <c r="BB2" t="inlineStr">
+        <is>
+          <t>UNLEADED 87 (10% ETH)</t>
+        </is>
+      </c>
+      <c r="BC2" t="inlineStr">
+        <is>
+          <t>2.899</t>
+        </is>
+      </c>
+      <c r="BD2" t="inlineStr">
+        <is>
+          <t>UNLEADED 87 (10% ETH)</t>
+        </is>
+      </c>
+      <c r="BE2" t="inlineStr">
+        <is>
+          <t>2.899</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1018,6 +1198,96 @@
           <t>$2.72</t>
         </is>
       </c>
+      <c r="AN3" t="inlineStr">
+        <is>
+          <t>That's Smart! Fat Free Skim Milk</t>
+        </is>
+      </c>
+      <c r="AO3" t="inlineStr">
+        <is>
+          <t>$2.72</t>
+        </is>
+      </c>
+      <c r="AP3" t="inlineStr">
+        <is>
+          <t>That's Smart! Fat Free Skim Milk</t>
+        </is>
+      </c>
+      <c r="AQ3" t="inlineStr">
+        <is>
+          <t>$2.72</t>
+        </is>
+      </c>
+      <c r="AR3" t="inlineStr">
+        <is>
+          <t>That's Smart! Fat Free Skim Milk</t>
+        </is>
+      </c>
+      <c r="AS3" t="inlineStr">
+        <is>
+          <t>$2.72</t>
+        </is>
+      </c>
+      <c r="AT3" t="inlineStr">
+        <is>
+          <t>That's Smart! Fat Free Skim Milk</t>
+        </is>
+      </c>
+      <c r="AU3" t="inlineStr">
+        <is>
+          <t>$2.72</t>
+        </is>
+      </c>
+      <c r="AV3" t="inlineStr">
+        <is>
+          <t>That's Smart! Fat Free Skim Milk</t>
+        </is>
+      </c>
+      <c r="AW3" t="inlineStr">
+        <is>
+          <t>$2.72</t>
+        </is>
+      </c>
+      <c r="AX3" t="inlineStr">
+        <is>
+          <t>That's Smart! Fat Free Skim Milk</t>
+        </is>
+      </c>
+      <c r="AY3" t="inlineStr">
+        <is>
+          <t>$2.72</t>
+        </is>
+      </c>
+      <c r="AZ3" t="inlineStr">
+        <is>
+          <t>That's Smart! Fat Free Skim Milk</t>
+        </is>
+      </c>
+      <c r="BA3" t="inlineStr">
+        <is>
+          <t>$2.72</t>
+        </is>
+      </c>
+      <c r="BB3" t="inlineStr">
+        <is>
+          <t>That's Smart! Fat Free Skim Milk</t>
+        </is>
+      </c>
+      <c r="BC3" t="inlineStr">
+        <is>
+          <t>$2.72</t>
+        </is>
+      </c>
+      <c r="BD3" t="inlineStr">
+        <is>
+          <t>That's Smart! Fat Free Skim Milk</t>
+        </is>
+      </c>
+      <c r="BE3" t="inlineStr">
+        <is>
+          <t>$2.72</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1215,6 +1485,96 @@
           <t>32¢ ea.</t>
         </is>
       </c>
+      <c r="AN4" t="inlineStr">
+        <is>
+          <t>Roma Tomatoes</t>
+        </is>
+      </c>
+      <c r="AO4" t="inlineStr">
+        <is>
+          <t>32¢ ea.</t>
+        </is>
+      </c>
+      <c r="AP4" t="inlineStr">
+        <is>
+          <t>Roma Tomatoes</t>
+        </is>
+      </c>
+      <c r="AQ4" t="inlineStr">
+        <is>
+          <t>32¢ ea.</t>
+        </is>
+      </c>
+      <c r="AR4" t="inlineStr">
+        <is>
+          <t>Roma Tomatoes</t>
+        </is>
+      </c>
+      <c r="AS4" t="inlineStr">
+        <is>
+          <t>32¢ ea.</t>
+        </is>
+      </c>
+      <c r="AT4" t="inlineStr">
+        <is>
+          <t>Roma Tomatoes</t>
+        </is>
+      </c>
+      <c r="AU4" t="inlineStr">
+        <is>
+          <t>32¢ ea.</t>
+        </is>
+      </c>
+      <c r="AV4" t="inlineStr">
+        <is>
+          <t>Roma Tomatoes</t>
+        </is>
+      </c>
+      <c r="AW4" t="inlineStr">
+        <is>
+          <t>32¢ ea.</t>
+        </is>
+      </c>
+      <c r="AX4" t="inlineStr">
+        <is>
+          <t>Roma Tomatoes</t>
+        </is>
+      </c>
+      <c r="AY4" t="inlineStr">
+        <is>
+          <t>38¢ ea.</t>
+        </is>
+      </c>
+      <c r="AZ4" t="inlineStr">
+        <is>
+          <t>Roma Tomatoes</t>
+        </is>
+      </c>
+      <c r="BA4" t="inlineStr">
+        <is>
+          <t>38¢ ea.</t>
+        </is>
+      </c>
+      <c r="BB4" t="inlineStr">
+        <is>
+          <t>Roma Tomatoes</t>
+        </is>
+      </c>
+      <c r="BC4" t="inlineStr">
+        <is>
+          <t>38¢ ea.</t>
+        </is>
+      </c>
+      <c r="BD4" t="inlineStr">
+        <is>
+          <t>Roma Tomatoes</t>
+        </is>
+      </c>
+      <c r="BE4" t="inlineStr">
+        <is>
+          <t>38¢ ea.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1412,6 +1772,96 @@
           <t>$4.97</t>
         </is>
       </c>
+      <c r="AN5" t="inlineStr">
+        <is>
+          <t>Quaker Cap'n Crunch Regular Cereal</t>
+        </is>
+      </c>
+      <c r="AO5" t="inlineStr">
+        <is>
+          <t>$4.97</t>
+        </is>
+      </c>
+      <c r="AP5" t="inlineStr">
+        <is>
+          <t>Quaker Cap'n Crunch Regular Cereal</t>
+        </is>
+      </c>
+      <c r="AQ5" t="inlineStr">
+        <is>
+          <t>$4.97</t>
+        </is>
+      </c>
+      <c r="AR5" t="inlineStr">
+        <is>
+          <t>Quaker Cap'n Crunch Regular Cereal</t>
+        </is>
+      </c>
+      <c r="AS5" t="inlineStr">
+        <is>
+          <t>$4.97</t>
+        </is>
+      </c>
+      <c r="AT5" t="inlineStr">
+        <is>
+          <t>Quaker Cap'n Crunch Regular Cereal</t>
+        </is>
+      </c>
+      <c r="AU5" t="inlineStr">
+        <is>
+          <t>$4.97</t>
+        </is>
+      </c>
+      <c r="AV5" t="inlineStr">
+        <is>
+          <t>Quaker Cap'n Crunch Regular Cereal</t>
+        </is>
+      </c>
+      <c r="AW5" t="inlineStr">
+        <is>
+          <t>$4.97</t>
+        </is>
+      </c>
+      <c r="AX5" t="inlineStr">
+        <is>
+          <t>Quaker Cap'n Crunch Regular Cereal</t>
+        </is>
+      </c>
+      <c r="AY5" t="inlineStr">
+        <is>
+          <t>$4.97</t>
+        </is>
+      </c>
+      <c r="AZ5" t="inlineStr">
+        <is>
+          <t>Quaker Cap'n Crunch Regular Cereal</t>
+        </is>
+      </c>
+      <c r="BA5" t="inlineStr">
+        <is>
+          <t>$4.97</t>
+        </is>
+      </c>
+      <c r="BB5" t="inlineStr">
+        <is>
+          <t>Quaker Cap'n Crunch Regular Cereal</t>
+        </is>
+      </c>
+      <c r="BC5" t="inlineStr">
+        <is>
+          <t>$4.97</t>
+        </is>
+      </c>
+      <c r="BD5" t="inlineStr">
+        <is>
+          <t>Quaker Cap'n Crunch Regular Cereal</t>
+        </is>
+      </c>
+      <c r="BE5" t="inlineStr">
+        <is>
+          <t>$4.97</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1609,6 +2059,96 @@
           <t>$3.99</t>
         </is>
       </c>
+      <c r="AN6" t="inlineStr">
+        <is>
+          <t>Sara Lee Artesano Brioche Buns, 8 count</t>
+        </is>
+      </c>
+      <c r="AO6" t="inlineStr">
+        <is>
+          <t>$3.99</t>
+        </is>
+      </c>
+      <c r="AP6" t="inlineStr">
+        <is>
+          <t>Sara Lee Artesano Brioche Buns, 8 count</t>
+        </is>
+      </c>
+      <c r="AQ6" t="inlineStr">
+        <is>
+          <t>$3.99</t>
+        </is>
+      </c>
+      <c r="AR6" t="inlineStr">
+        <is>
+          <t>Sara Lee Artesano Brioche Buns, 8 count</t>
+        </is>
+      </c>
+      <c r="AS6" t="inlineStr">
+        <is>
+          <t>$3.99</t>
+        </is>
+      </c>
+      <c r="AT6" t="inlineStr">
+        <is>
+          <t>Sara Lee Artesano Brioche Buns, 8 count</t>
+        </is>
+      </c>
+      <c r="AU6" t="inlineStr">
+        <is>
+          <t>$3.99</t>
+        </is>
+      </c>
+      <c r="AV6" t="inlineStr">
+        <is>
+          <t>Sara Lee Artesano Brioche Buns, 8 count</t>
+        </is>
+      </c>
+      <c r="AW6" t="inlineStr">
+        <is>
+          <t>$3.99</t>
+        </is>
+      </c>
+      <c r="AX6" t="inlineStr">
+        <is>
+          <t>Sara Lee Artesano Brioche Buns, 8 count</t>
+        </is>
+      </c>
+      <c r="AY6" t="inlineStr">
+        <is>
+          <t>$3.99</t>
+        </is>
+      </c>
+      <c r="AZ6" t="inlineStr">
+        <is>
+          <t>Sara Lee Artesano Brioche Buns, 8 count</t>
+        </is>
+      </c>
+      <c r="BA6" t="inlineStr">
+        <is>
+          <t>$3.99</t>
+        </is>
+      </c>
+      <c r="BB6" t="inlineStr">
+        <is>
+          <t>Sara Lee Artesano Brioche Buns, 8 count</t>
+        </is>
+      </c>
+      <c r="BC6" t="inlineStr">
+        <is>
+          <t>$3.99</t>
+        </is>
+      </c>
+      <c r="BD6" t="inlineStr">
+        <is>
+          <t>Sara Lee Artesano Brioche Buns, 8 count</t>
+        </is>
+      </c>
+      <c r="BE6" t="inlineStr">
+        <is>
+          <t>$3.99</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1806,6 +2346,96 @@
           <t>$3.65</t>
         </is>
       </c>
+      <c r="AN7" t="inlineStr">
+        <is>
+          <t>That's Smart! Mayonnaise</t>
+        </is>
+      </c>
+      <c r="AO7" t="inlineStr">
+        <is>
+          <t>$3.65</t>
+        </is>
+      </c>
+      <c r="AP7" t="inlineStr">
+        <is>
+          <t>That's Smart! Mayonnaise</t>
+        </is>
+      </c>
+      <c r="AQ7" t="inlineStr">
+        <is>
+          <t>$3.65</t>
+        </is>
+      </c>
+      <c r="AR7" t="inlineStr">
+        <is>
+          <t>That's Smart! Mayonnaise</t>
+        </is>
+      </c>
+      <c r="AS7" t="inlineStr">
+        <is>
+          <t>$3.65</t>
+        </is>
+      </c>
+      <c r="AT7" t="inlineStr">
+        <is>
+          <t>That's Smart! Mayonnaise</t>
+        </is>
+      </c>
+      <c r="AU7" t="inlineStr">
+        <is>
+          <t>$3.65</t>
+        </is>
+      </c>
+      <c r="AV7" t="inlineStr">
+        <is>
+          <t>That's Smart! Mayonnaise</t>
+        </is>
+      </c>
+      <c r="AW7" t="inlineStr">
+        <is>
+          <t>$3.65</t>
+        </is>
+      </c>
+      <c r="AX7" t="inlineStr">
+        <is>
+          <t>That's Smart! Mayonnaise</t>
+        </is>
+      </c>
+      <c r="AY7" t="inlineStr">
+        <is>
+          <t>$3.65</t>
+        </is>
+      </c>
+      <c r="AZ7" t="inlineStr">
+        <is>
+          <t>That's Smart! Mayonnaise</t>
+        </is>
+      </c>
+      <c r="BA7" t="inlineStr">
+        <is>
+          <t>$3.65</t>
+        </is>
+      </c>
+      <c r="BB7" t="inlineStr">
+        <is>
+          <t>That's Smart! Mayonnaise</t>
+        </is>
+      </c>
+      <c r="BC7" t="inlineStr">
+        <is>
+          <t>$3.65</t>
+        </is>
+      </c>
+      <c r="BD7" t="inlineStr">
+        <is>
+          <t>That's Smart! Mayonnaise</t>
+        </is>
+      </c>
+      <c r="BE7" t="inlineStr">
+        <is>
+          <t>$3.65</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -2003,6 +2633,96 @@
           <t>$1.99</t>
         </is>
       </c>
+      <c r="AN8" t="inlineStr">
+        <is>
+          <t>Hy-Vee Light Bartlett Pear Halves In Pear Juice From Concentrate</t>
+        </is>
+      </c>
+      <c r="AO8" t="inlineStr">
+        <is>
+          <t>$1.99</t>
+        </is>
+      </c>
+      <c r="AP8" t="inlineStr">
+        <is>
+          <t>Hy-Vee Light Bartlett Pear Halves In Pear Juice From Concentrate</t>
+        </is>
+      </c>
+      <c r="AQ8" t="inlineStr">
+        <is>
+          <t>$1.99</t>
+        </is>
+      </c>
+      <c r="AR8" t="inlineStr">
+        <is>
+          <t>Hy-Vee Light Bartlett Pear Halves In Pear Juice From Concentrate</t>
+        </is>
+      </c>
+      <c r="AS8" t="inlineStr">
+        <is>
+          <t>$1.99</t>
+        </is>
+      </c>
+      <c r="AT8" t="inlineStr">
+        <is>
+          <t>Hy-Vee Light Bartlett Pear Halves In Pear Juice From Concentrate</t>
+        </is>
+      </c>
+      <c r="AU8" t="inlineStr">
+        <is>
+          <t>$1.99</t>
+        </is>
+      </c>
+      <c r="AV8" t="inlineStr">
+        <is>
+          <t>Hy-Vee Light Bartlett Pear Halves In Pear Juice From Concentrate</t>
+        </is>
+      </c>
+      <c r="AW8" t="inlineStr">
+        <is>
+          <t>$1.99</t>
+        </is>
+      </c>
+      <c r="AX8" t="inlineStr">
+        <is>
+          <t>Hy-Vee Light Bartlett Pear Halves In Pear Juice From Concentrate</t>
+        </is>
+      </c>
+      <c r="AY8" t="inlineStr">
+        <is>
+          <t>$1.99</t>
+        </is>
+      </c>
+      <c r="AZ8" t="inlineStr">
+        <is>
+          <t>Hy-Vee Light Bartlett Pear Halves In Pear Juice From Concentrate</t>
+        </is>
+      </c>
+      <c r="BA8" t="inlineStr">
+        <is>
+          <t>$1.99</t>
+        </is>
+      </c>
+      <c r="BB8" t="inlineStr">
+        <is>
+          <t>Hy-Vee Light Bartlett Pear Halves In Pear Juice From Concentrate</t>
+        </is>
+      </c>
+      <c r="BC8" t="inlineStr">
+        <is>
+          <t>$1.99</t>
+        </is>
+      </c>
+      <c r="BD8" t="inlineStr">
+        <is>
+          <t>Hy-Vee Light Bartlett Pear Halves In Pear Juice From Concentrate</t>
+        </is>
+      </c>
+      <c r="BE8" t="inlineStr">
+        <is>
+          <t>$1.99</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -2200,6 +2920,96 @@
           <t>$3.99</t>
         </is>
       </c>
+      <c r="AN9" t="inlineStr">
+        <is>
+          <t>Dole Fresh Romaine Hearts</t>
+        </is>
+      </c>
+      <c r="AO9" t="inlineStr">
+        <is>
+          <t>$3.99</t>
+        </is>
+      </c>
+      <c r="AP9" t="inlineStr">
+        <is>
+          <t>Dole Fresh Romaine Hearts</t>
+        </is>
+      </c>
+      <c r="AQ9" t="inlineStr">
+        <is>
+          <t>$3.99</t>
+        </is>
+      </c>
+      <c r="AR9" t="inlineStr">
+        <is>
+          <t>Dole Fresh Romaine Hearts</t>
+        </is>
+      </c>
+      <c r="AS9" t="inlineStr">
+        <is>
+          <t>$3.99</t>
+        </is>
+      </c>
+      <c r="AT9" t="inlineStr">
+        <is>
+          <t>Dole Fresh Romaine Hearts</t>
+        </is>
+      </c>
+      <c r="AU9" t="inlineStr">
+        <is>
+          <t>$3.99</t>
+        </is>
+      </c>
+      <c r="AV9" t="inlineStr">
+        <is>
+          <t>Dole Fresh Romaine Hearts</t>
+        </is>
+      </c>
+      <c r="AW9" t="inlineStr">
+        <is>
+          <t>$3.99</t>
+        </is>
+      </c>
+      <c r="AX9" t="inlineStr">
+        <is>
+          <t>Dole Fresh Romaine Hearts</t>
+        </is>
+      </c>
+      <c r="AY9" t="inlineStr">
+        <is>
+          <t>$3.99</t>
+        </is>
+      </c>
+      <c r="AZ9" t="inlineStr">
+        <is>
+          <t>Dole Fresh Romaine Hearts</t>
+        </is>
+      </c>
+      <c r="BA9" t="inlineStr">
+        <is>
+          <t>$3.99</t>
+        </is>
+      </c>
+      <c r="BB9" t="inlineStr">
+        <is>
+          <t>Dole Fresh Romaine Hearts</t>
+        </is>
+      </c>
+      <c r="BC9" t="inlineStr">
+        <is>
+          <t>$3.99</t>
+        </is>
+      </c>
+      <c r="BD9" t="inlineStr">
+        <is>
+          <t>Dole Fresh Romaine Hearts</t>
+        </is>
+      </c>
+      <c r="BE9" t="inlineStr">
+        <is>
+          <t>$3.99</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -2397,6 +3207,96 @@
           <t>$5.79</t>
         </is>
       </c>
+      <c r="AN10" t="inlineStr">
+        <is>
+          <t>Hy-Vee Oven Roasted Cured Turkey Breast &amp; White Turkey Shaved Slices</t>
+        </is>
+      </c>
+      <c r="AO10" t="inlineStr">
+        <is>
+          <t>$5.79</t>
+        </is>
+      </c>
+      <c r="AP10" t="inlineStr">
+        <is>
+          <t>Hy-Vee Oven Roasted Cured Turkey Breast &amp; White Turkey Shaved Slices</t>
+        </is>
+      </c>
+      <c r="AQ10" t="inlineStr">
+        <is>
+          <t>$5.79</t>
+        </is>
+      </c>
+      <c r="AR10" t="inlineStr">
+        <is>
+          <t>Hy-Vee Oven Roasted Cured Turkey Breast &amp; White Turkey Shaved Slices</t>
+        </is>
+      </c>
+      <c r="AS10" t="inlineStr">
+        <is>
+          <t>$5.79</t>
+        </is>
+      </c>
+      <c r="AT10" t="inlineStr">
+        <is>
+          <t>Hy-Vee Oven Roasted Cured Turkey Breast &amp; White Turkey Shaved Slices</t>
+        </is>
+      </c>
+      <c r="AU10" t="inlineStr">
+        <is>
+          <t>$5.79</t>
+        </is>
+      </c>
+      <c r="AV10" t="inlineStr">
+        <is>
+          <t>Hy-Vee Oven Roasted Cured Turkey Breast &amp; White Turkey Shaved Slices</t>
+        </is>
+      </c>
+      <c r="AW10" t="inlineStr">
+        <is>
+          <t>$5.79</t>
+        </is>
+      </c>
+      <c r="AX10" t="inlineStr">
+        <is>
+          <t>Hy-Vee Oven Roasted Cured Turkey Breast &amp; White Turkey Shaved Slices</t>
+        </is>
+      </c>
+      <c r="AY10" t="inlineStr">
+        <is>
+          <t>$5.79</t>
+        </is>
+      </c>
+      <c r="AZ10" t="inlineStr">
+        <is>
+          <t>Hy-Vee Oven Roasted Cured Turkey Breast &amp; White Turkey Shaved Slices</t>
+        </is>
+      </c>
+      <c r="BA10" t="inlineStr">
+        <is>
+          <t>$5.79</t>
+        </is>
+      </c>
+      <c r="BB10" t="inlineStr">
+        <is>
+          <t>Hy-Vee Oven Roasted Cured Turkey Breast &amp; White Turkey Shaved Slices</t>
+        </is>
+      </c>
+      <c r="BC10" t="inlineStr">
+        <is>
+          <t>$5.79</t>
+        </is>
+      </c>
+      <c r="BD10" t="inlineStr">
+        <is>
+          <t>Hy-Vee Oven Roasted Cured Turkey Breast &amp; White Turkey Shaved Slices</t>
+        </is>
+      </c>
+      <c r="BE10" t="inlineStr">
+        <is>
+          <t>$5.79</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -2594,6 +3494,96 @@
           <t>$2.99</t>
         </is>
       </c>
+      <c r="AN11" t="inlineStr">
+        <is>
+          <t>That's Smart! Small Curd Cottage Cheese 4% Milkfat</t>
+        </is>
+      </c>
+      <c r="AO11" t="inlineStr">
+        <is>
+          <t>$2.99</t>
+        </is>
+      </c>
+      <c r="AP11" t="inlineStr">
+        <is>
+          <t>That's Smart! Small Curd Cottage Cheese 4% Milkfat</t>
+        </is>
+      </c>
+      <c r="AQ11" t="inlineStr">
+        <is>
+          <t>$2.99</t>
+        </is>
+      </c>
+      <c r="AR11" t="inlineStr">
+        <is>
+          <t>That's Smart! Small Curd Cottage Cheese 4% Milkfat</t>
+        </is>
+      </c>
+      <c r="AS11" t="inlineStr">
+        <is>
+          <t>$2.99</t>
+        </is>
+      </c>
+      <c r="AT11" t="inlineStr">
+        <is>
+          <t>That's Smart! Small Curd Cottage Cheese 4% Milkfat</t>
+        </is>
+      </c>
+      <c r="AU11" t="inlineStr">
+        <is>
+          <t>$2.99</t>
+        </is>
+      </c>
+      <c r="AV11" t="inlineStr">
+        <is>
+          <t>That's Smart! Small Curd Cottage Cheese 4% Milkfat</t>
+        </is>
+      </c>
+      <c r="AW11" t="inlineStr">
+        <is>
+          <t>$2.99</t>
+        </is>
+      </c>
+      <c r="AX11" t="inlineStr">
+        <is>
+          <t>That's Smart! Small Curd Cottage Cheese 4% Milkfat</t>
+        </is>
+      </c>
+      <c r="AY11" t="inlineStr">
+        <is>
+          <t>$2.99</t>
+        </is>
+      </c>
+      <c r="AZ11" t="inlineStr">
+        <is>
+          <t>That's Smart! Small Curd Cottage Cheese 4% Milkfat</t>
+        </is>
+      </c>
+      <c r="BA11" t="inlineStr">
+        <is>
+          <t>$2.99</t>
+        </is>
+      </c>
+      <c r="BB11" t="inlineStr">
+        <is>
+          <t>That's Smart! Small Curd Cottage Cheese 4% Milkfat</t>
+        </is>
+      </c>
+      <c r="BC11" t="inlineStr">
+        <is>
+          <t>$2.99</t>
+        </is>
+      </c>
+      <c r="BD11" t="inlineStr">
+        <is>
+          <t>That's Smart! Small Curd Cottage Cheese 4% Milkfat</t>
+        </is>
+      </c>
+      <c r="BE11" t="inlineStr">
+        <is>
+          <t>$2.99</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -2791,6 +3781,96 @@
           <t>$4.97</t>
         </is>
       </c>
+      <c r="AN12" t="inlineStr">
+        <is>
+          <t>Fairlife Fat Free Ultra-Filtered Milk</t>
+        </is>
+      </c>
+      <c r="AO12" t="inlineStr">
+        <is>
+          <t>$4.97</t>
+        </is>
+      </c>
+      <c r="AP12" t="inlineStr">
+        <is>
+          <t>Fairlife Fat Free Ultra-Filtered Milk</t>
+        </is>
+      </c>
+      <c r="AQ12" t="inlineStr">
+        <is>
+          <t>$4.97</t>
+        </is>
+      </c>
+      <c r="AR12" t="inlineStr">
+        <is>
+          <t>Fairlife Fat Free Ultra-Filtered Milk</t>
+        </is>
+      </c>
+      <c r="AS12" t="inlineStr">
+        <is>
+          <t>$4.97</t>
+        </is>
+      </c>
+      <c r="AT12" t="inlineStr">
+        <is>
+          <t>Fairlife Fat Free Ultra-Filtered Milk</t>
+        </is>
+      </c>
+      <c r="AU12" t="inlineStr">
+        <is>
+          <t>$4.97</t>
+        </is>
+      </c>
+      <c r="AV12" t="inlineStr">
+        <is>
+          <t>Fairlife Fat Free Ultra-Filtered Milk</t>
+        </is>
+      </c>
+      <c r="AW12" t="inlineStr">
+        <is>
+          <t>$4.97</t>
+        </is>
+      </c>
+      <c r="AX12" t="inlineStr">
+        <is>
+          <t>Fairlife Fat Free Ultra-Filtered Milk</t>
+        </is>
+      </c>
+      <c r="AY12" t="inlineStr">
+        <is>
+          <t>$4.97</t>
+        </is>
+      </c>
+      <c r="AZ12" t="inlineStr">
+        <is>
+          <t>Fairlife Fat Free Ultra-Filtered Milk</t>
+        </is>
+      </c>
+      <c r="BA12" t="inlineStr">
+        <is>
+          <t>$4.97</t>
+        </is>
+      </c>
+      <c r="BB12" t="inlineStr">
+        <is>
+          <t>Fairlife Fat Free Ultra-Filtered Milk</t>
+        </is>
+      </c>
+      <c r="BC12" t="inlineStr">
+        <is>
+          <t>$4.97</t>
+        </is>
+      </c>
+      <c r="BD12" t="inlineStr">
+        <is>
+          <t>Fairlife Fat Free Ultra-Filtered Milk</t>
+        </is>
+      </c>
+      <c r="BE12" t="inlineStr">
+        <is>
+          <t>$4.97</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -2988,6 +4068,96 @@
           <t>16¢ ea.</t>
         </is>
       </c>
+      <c r="AN13" t="inlineStr">
+        <is>
+          <t>Fresh Chiquita Bananas</t>
+        </is>
+      </c>
+      <c r="AO13" t="inlineStr">
+        <is>
+          <t>16¢ ea.</t>
+        </is>
+      </c>
+      <c r="AP13" t="inlineStr">
+        <is>
+          <t>Fresh Chiquita Bananas</t>
+        </is>
+      </c>
+      <c r="AQ13" t="inlineStr">
+        <is>
+          <t>16¢ ea.</t>
+        </is>
+      </c>
+      <c r="AR13" t="inlineStr">
+        <is>
+          <t>Fresh Chiquita Bananas</t>
+        </is>
+      </c>
+      <c r="AS13" t="inlineStr">
+        <is>
+          <t>16¢ ea.</t>
+        </is>
+      </c>
+      <c r="AT13" t="inlineStr">
+        <is>
+          <t>Fresh Chiquita Bananas</t>
+        </is>
+      </c>
+      <c r="AU13" t="inlineStr">
+        <is>
+          <t>16¢ ea.</t>
+        </is>
+      </c>
+      <c r="AV13" t="inlineStr">
+        <is>
+          <t>Fresh Chiquita Bananas</t>
+        </is>
+      </c>
+      <c r="AW13" t="inlineStr">
+        <is>
+          <t>16¢ ea.</t>
+        </is>
+      </c>
+      <c r="AX13" t="inlineStr">
+        <is>
+          <t>Fresh Chiquita Bananas</t>
+        </is>
+      </c>
+      <c r="AY13" t="inlineStr">
+        <is>
+          <t>16¢ ea.</t>
+        </is>
+      </c>
+      <c r="AZ13" t="inlineStr">
+        <is>
+          <t>Fresh Chiquita Bananas</t>
+        </is>
+      </c>
+      <c r="BA13" t="inlineStr">
+        <is>
+          <t>16¢ ea.</t>
+        </is>
+      </c>
+      <c r="BB13" t="inlineStr">
+        <is>
+          <t>Fresh Chiquita Bananas</t>
+        </is>
+      </c>
+      <c r="BC13" t="inlineStr">
+        <is>
+          <t>16¢ ea.</t>
+        </is>
+      </c>
+      <c r="BD13" t="inlineStr">
+        <is>
+          <t>Fresh Chiquita Bananas</t>
+        </is>
+      </c>
+      <c r="BE13" t="inlineStr">
+        <is>
+          <t>16¢ ea.</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -3185,6 +4355,96 @@
           <t>$4.99</t>
         </is>
       </c>
+      <c r="AN14" t="inlineStr">
+        <is>
+          <t>Wonderful Halos Mandarin Oranges</t>
+        </is>
+      </c>
+      <c r="AO14" t="inlineStr">
+        <is>
+          <t>$4.99</t>
+        </is>
+      </c>
+      <c r="AP14" t="inlineStr">
+        <is>
+          <t>Wonderful Halos Mandarin Oranges</t>
+        </is>
+      </c>
+      <c r="AQ14" t="inlineStr">
+        <is>
+          <t>$4.99</t>
+        </is>
+      </c>
+      <c r="AR14" t="inlineStr">
+        <is>
+          <t>Wonderful Halos Mandarin Oranges</t>
+        </is>
+      </c>
+      <c r="AS14" t="inlineStr">
+        <is>
+          <t>$4.99</t>
+        </is>
+      </c>
+      <c r="AT14" t="inlineStr">
+        <is>
+          <t>Wonderful Halos Mandarin Oranges</t>
+        </is>
+      </c>
+      <c r="AU14" t="inlineStr">
+        <is>
+          <t>$4.99</t>
+        </is>
+      </c>
+      <c r="AV14" t="inlineStr">
+        <is>
+          <t>Wonderful Halos Mandarin Oranges</t>
+        </is>
+      </c>
+      <c r="AW14" t="inlineStr">
+        <is>
+          <t>$4.99</t>
+        </is>
+      </c>
+      <c r="AX14" t="inlineStr">
+        <is>
+          <t>Wonderful Halos Mandarin Oranges</t>
+        </is>
+      </c>
+      <c r="AY14" t="inlineStr">
+        <is>
+          <t>$5.89</t>
+        </is>
+      </c>
+      <c r="AZ14" t="inlineStr">
+        <is>
+          <t>Wonderful Halos Mandarin Oranges</t>
+        </is>
+      </c>
+      <c r="BA14" t="inlineStr">
+        <is>
+          <t>$5.89</t>
+        </is>
+      </c>
+      <c r="BB14" t="inlineStr">
+        <is>
+          <t>Wonderful Halos Mandarin Oranges</t>
+        </is>
+      </c>
+      <c r="BC14" t="inlineStr">
+        <is>
+          <t>$5.89</t>
+        </is>
+      </c>
+      <c r="BD14" t="inlineStr">
+        <is>
+          <t>Wonderful Halos Mandarin Oranges</t>
+        </is>
+      </c>
+      <c r="BE14" t="inlineStr">
+        <is>
+          <t>$5.89</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -3382,6 +4642,96 @@
           <t>$6.99/lb</t>
         </is>
       </c>
+      <c r="AN15" t="inlineStr">
+        <is>
+          <t>Certified Ground Round 90% Lean 10% Fat</t>
+        </is>
+      </c>
+      <c r="AO15" t="inlineStr">
+        <is>
+          <t>$6.99/lb</t>
+        </is>
+      </c>
+      <c r="AP15" t="inlineStr">
+        <is>
+          <t>Certified Ground Round 90% Lean 10% Fat</t>
+        </is>
+      </c>
+      <c r="AQ15" t="inlineStr">
+        <is>
+          <t>$6.99/lb</t>
+        </is>
+      </c>
+      <c r="AR15" t="inlineStr">
+        <is>
+          <t>Certified Ground Round 90% Lean 10% Fat</t>
+        </is>
+      </c>
+      <c r="AS15" t="inlineStr">
+        <is>
+          <t>$6.99/lb</t>
+        </is>
+      </c>
+      <c r="AT15" t="inlineStr">
+        <is>
+          <t>Certified Ground Round 90% Lean 10% Fat</t>
+        </is>
+      </c>
+      <c r="AU15" t="inlineStr">
+        <is>
+          <t>$6.99/lb</t>
+        </is>
+      </c>
+      <c r="AV15" t="inlineStr">
+        <is>
+          <t>Certified Ground Round 90% Lean 10% Fat</t>
+        </is>
+      </c>
+      <c r="AW15" t="inlineStr">
+        <is>
+          <t>$6.99/lb</t>
+        </is>
+      </c>
+      <c r="AX15" t="inlineStr">
+        <is>
+          <t>Certified Ground Round 90% Lean 10% Fat</t>
+        </is>
+      </c>
+      <c r="AY15" t="inlineStr">
+        <is>
+          <t>$6.99/lb</t>
+        </is>
+      </c>
+      <c r="AZ15" t="inlineStr">
+        <is>
+          <t>Certified Ground Round 90% Lean 10% Fat</t>
+        </is>
+      </c>
+      <c r="BA15" t="inlineStr">
+        <is>
+          <t>$6.99/lb</t>
+        </is>
+      </c>
+      <c r="BB15" t="inlineStr">
+        <is>
+          <t>Certified Ground Round 90% Lean 10% Fat</t>
+        </is>
+      </c>
+      <c r="BC15" t="inlineStr">
+        <is>
+          <t>$6.99/lb</t>
+        </is>
+      </c>
+      <c r="BD15" t="inlineStr">
+        <is>
+          <t>Certified Ground Round 90% Lean 10% Fat</t>
+        </is>
+      </c>
+      <c r="BE15" t="inlineStr">
+        <is>
+          <t>$6.99/lb</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -3579,6 +4929,96 @@
           <t>$3.19 ea.</t>
         </is>
       </c>
+      <c r="AN16" t="inlineStr">
+        <is>
+          <t>Boneless Skinless Chicken Breast</t>
+        </is>
+      </c>
+      <c r="AO16" t="inlineStr">
+        <is>
+          <t>$3.19 ea.</t>
+        </is>
+      </c>
+      <c r="AP16" t="inlineStr">
+        <is>
+          <t>Boneless Skinless Chicken Breast</t>
+        </is>
+      </c>
+      <c r="AQ16" t="inlineStr">
+        <is>
+          <t>$3.19 ea.</t>
+        </is>
+      </c>
+      <c r="AR16" t="inlineStr">
+        <is>
+          <t>Boneless Skinless Chicken Breast</t>
+        </is>
+      </c>
+      <c r="AS16" t="inlineStr">
+        <is>
+          <t>$3.19 ea.</t>
+        </is>
+      </c>
+      <c r="AT16" t="inlineStr">
+        <is>
+          <t>Boneless Skinless Chicken Breast</t>
+        </is>
+      </c>
+      <c r="AU16" t="inlineStr">
+        <is>
+          <t>$3.19 ea.</t>
+        </is>
+      </c>
+      <c r="AV16" t="inlineStr">
+        <is>
+          <t>Boneless Skinless Chicken Breast</t>
+        </is>
+      </c>
+      <c r="AW16" t="inlineStr">
+        <is>
+          <t>$3.19 ea.</t>
+        </is>
+      </c>
+      <c r="AX16" t="inlineStr">
+        <is>
+          <t>Boneless Skinless Chicken Breast</t>
+        </is>
+      </c>
+      <c r="AY16" t="inlineStr">
+        <is>
+          <t>$3.19 ea.</t>
+        </is>
+      </c>
+      <c r="AZ16" t="inlineStr">
+        <is>
+          <t>Boneless Skinless Chicken Breast</t>
+        </is>
+      </c>
+      <c r="BA16" t="inlineStr">
+        <is>
+          <t>$3.83 ea.</t>
+        </is>
+      </c>
+      <c r="BB16" t="inlineStr">
+        <is>
+          <t>Boneless Skinless Chicken Breast</t>
+        </is>
+      </c>
+      <c r="BC16" t="inlineStr">
+        <is>
+          <t>$3.83 ea.</t>
+        </is>
+      </c>
+      <c r="BD16" t="inlineStr">
+        <is>
+          <t>Boneless Skinless Chicken Breast</t>
+        </is>
+      </c>
+      <c r="BE16" t="inlineStr">
+        <is>
+          <t>$3.83 ea.</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -3776,6 +5216,96 @@
           <t>$40,275</t>
         </is>
       </c>
+      <c r="AN17" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="AO17" t="inlineStr">
+        <is>
+          <t>$40,275</t>
+        </is>
+      </c>
+      <c r="AP17" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="AQ17" t="inlineStr">
+        <is>
+          <t>$40,275</t>
+        </is>
+      </c>
+      <c r="AR17" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="AS17" t="inlineStr">
+        <is>
+          <t>$40,275</t>
+        </is>
+      </c>
+      <c r="AT17" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="AU17" t="inlineStr">
+        <is>
+          <t>$40,275</t>
+        </is>
+      </c>
+      <c r="AV17" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="AW17" t="inlineStr">
+        <is>
+          <t>$40,275</t>
+        </is>
+      </c>
+      <c r="AX17" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="AY17" t="inlineStr">
+        <is>
+          <t>$40,275</t>
+        </is>
+      </c>
+      <c r="AZ17" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="BA17" t="inlineStr">
+        <is>
+          <t>$40,275</t>
+        </is>
+      </c>
+      <c r="BB17" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="BC17" t="inlineStr">
+        <is>
+          <t>$40,275</t>
+        </is>
+      </c>
+      <c r="BD17" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="BE17" t="inlineStr">
+        <is>
+          <t>$40,275</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -3893,6 +5423,60 @@
       </c>
       <c r="AL18" t="inlineStr"/>
       <c r="AM18" t="inlineStr">
+        <is>
+          <t>$37,000*</t>
+        </is>
+      </c>
+      <c r="AN18" t="inlineStr"/>
+      <c r="AO18" t="inlineStr">
+        <is>
+          <t>$37,000*</t>
+        </is>
+      </c>
+      <c r="AP18" t="inlineStr"/>
+      <c r="AQ18" t="inlineStr">
+        <is>
+          <t>$37,000*</t>
+        </is>
+      </c>
+      <c r="AR18" t="inlineStr"/>
+      <c r="AS18" t="inlineStr">
+        <is>
+          <t>$37,000*</t>
+        </is>
+      </c>
+      <c r="AT18" t="inlineStr"/>
+      <c r="AU18" t="inlineStr">
+        <is>
+          <t>$37,000*</t>
+        </is>
+      </c>
+      <c r="AV18" t="inlineStr"/>
+      <c r="AW18" t="inlineStr">
+        <is>
+          <t>$37,000*</t>
+        </is>
+      </c>
+      <c r="AX18" t="inlineStr"/>
+      <c r="AY18" t="inlineStr">
+        <is>
+          <t>$37,000*</t>
+        </is>
+      </c>
+      <c r="AZ18" t="inlineStr"/>
+      <c r="BA18" t="inlineStr">
+        <is>
+          <t>$37,000*</t>
+        </is>
+      </c>
+      <c r="BB18" t="inlineStr"/>
+      <c r="BC18" t="inlineStr">
+        <is>
+          <t>$37,000*</t>
+        </is>
+      </c>
+      <c r="BD18" t="inlineStr"/>
+      <c r="BE18" t="inlineStr">
         <is>
           <t>$37,000*</t>
         </is>
@@ -4046,6 +5630,60 @@
           <t>Not found</t>
         </is>
       </c>
+      <c r="AN19" t="inlineStr"/>
+      <c r="AO19" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="AP19" t="inlineStr"/>
+      <c r="AQ19" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="AR19" t="inlineStr"/>
+      <c r="AS19" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="AT19" t="inlineStr"/>
+      <c r="AU19" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="AV19" t="inlineStr"/>
+      <c r="AW19" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="AX19" t="inlineStr"/>
+      <c r="AY19" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="AZ19" t="inlineStr"/>
+      <c r="BA19" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="BB19" t="inlineStr"/>
+      <c r="BC19" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="BD19" t="inlineStr"/>
+      <c r="BE19" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -4243,6 +5881,96 @@
           <t>$6.99</t>
         </is>
       </c>
+      <c r="AN20" t="inlineStr">
+        <is>
+          <t>Hy-Vee Select 100% Pure Maple Syrup</t>
+        </is>
+      </c>
+      <c r="AO20" t="inlineStr">
+        <is>
+          <t>$6.99</t>
+        </is>
+      </c>
+      <c r="AP20" t="inlineStr">
+        <is>
+          <t>Hy-Vee Select 100% Pure Maple Syrup</t>
+        </is>
+      </c>
+      <c r="AQ20" t="inlineStr">
+        <is>
+          <t>$6.99</t>
+        </is>
+      </c>
+      <c r="AR20" t="inlineStr">
+        <is>
+          <t>Hy-Vee Select 100% Pure Maple Syrup</t>
+        </is>
+      </c>
+      <c r="AS20" t="inlineStr">
+        <is>
+          <t>$6.99</t>
+        </is>
+      </c>
+      <c r="AT20" t="inlineStr">
+        <is>
+          <t>Hy-Vee Select 100% Pure Maple Syrup</t>
+        </is>
+      </c>
+      <c r="AU20" t="inlineStr">
+        <is>
+          <t>$6.99</t>
+        </is>
+      </c>
+      <c r="AV20" t="inlineStr">
+        <is>
+          <t>Hy-Vee Select 100% Pure Maple Syrup</t>
+        </is>
+      </c>
+      <c r="AW20" t="inlineStr">
+        <is>
+          <t>$6.99</t>
+        </is>
+      </c>
+      <c r="AX20" t="inlineStr">
+        <is>
+          <t>Hy-Vee Select 100% Pure Maple Syrup</t>
+        </is>
+      </c>
+      <c r="AY20" t="inlineStr">
+        <is>
+          <t>$6.99</t>
+        </is>
+      </c>
+      <c r="AZ20" t="inlineStr">
+        <is>
+          <t>Hy-Vee Select 100% Pure Maple Syrup</t>
+        </is>
+      </c>
+      <c r="BA20" t="inlineStr">
+        <is>
+          <t>$6.99</t>
+        </is>
+      </c>
+      <c r="BB20" t="inlineStr">
+        <is>
+          <t>Hy-Vee Select 100% Pure Maple Syrup</t>
+        </is>
+      </c>
+      <c r="BC20" t="inlineStr">
+        <is>
+          <t>$6.99</t>
+        </is>
+      </c>
+      <c r="BD20" t="inlineStr">
+        <is>
+          <t>Hy-Vee Select 100% Pure Maple Syrup</t>
+        </is>
+      </c>
+      <c r="BE20" t="inlineStr">
+        <is>
+          <t>$6.99</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -4440,6 +6168,96 @@
           <t>$5.97</t>
         </is>
       </c>
+      <c r="AN21" t="inlineStr">
+        <is>
+          <t>That's Smart! Large Shell Eggs</t>
+        </is>
+      </c>
+      <c r="AO21" t="inlineStr">
+        <is>
+          <t>$5.97</t>
+        </is>
+      </c>
+      <c r="AP21" t="inlineStr">
+        <is>
+          <t>That's Smart! Large Shell Eggs</t>
+        </is>
+      </c>
+      <c r="AQ21" t="inlineStr">
+        <is>
+          <t>$5.97</t>
+        </is>
+      </c>
+      <c r="AR21" t="inlineStr">
+        <is>
+          <t>That's Smart! Large Shell Eggs</t>
+        </is>
+      </c>
+      <c r="AS21" t="inlineStr">
+        <is>
+          <t>$5.97</t>
+        </is>
+      </c>
+      <c r="AT21" t="inlineStr">
+        <is>
+          <t>That's Smart! Large Shell Eggs</t>
+        </is>
+      </c>
+      <c r="AU21" t="inlineStr">
+        <is>
+          <t>$5.97</t>
+        </is>
+      </c>
+      <c r="AV21" t="inlineStr">
+        <is>
+          <t>That's Smart! Large Shell Eggs</t>
+        </is>
+      </c>
+      <c r="AW21" t="inlineStr">
+        <is>
+          <t>$5.97</t>
+        </is>
+      </c>
+      <c r="AX21" t="inlineStr">
+        <is>
+          <t>That's Smart! Large Shell Eggs</t>
+        </is>
+      </c>
+      <c r="AY21" t="inlineStr">
+        <is>
+          <t>$5.97</t>
+        </is>
+      </c>
+      <c r="AZ21" t="inlineStr">
+        <is>
+          <t>That's Smart! Large Shell Eggs</t>
+        </is>
+      </c>
+      <c r="BA21" t="inlineStr">
+        <is>
+          <t>$5.97</t>
+        </is>
+      </c>
+      <c r="BB21" t="inlineStr">
+        <is>
+          <t>That's Smart! Large Shell Eggs</t>
+        </is>
+      </c>
+      <c r="BC21" t="inlineStr">
+        <is>
+          <t>$5.97</t>
+        </is>
+      </c>
+      <c r="BD21" t="inlineStr">
+        <is>
+          <t>That's Smart! Large Shell Eggs</t>
+        </is>
+      </c>
+      <c r="BE21" t="inlineStr">
+        <is>
+          <t>$5.97</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -4637,6 +6455,96 @@
           <t>698</t>
         </is>
       </c>
+      <c r="AN22" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="AO22" t="inlineStr">
+        <is>
+          <t>698</t>
+        </is>
+      </c>
+      <c r="AP22" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="AQ22" t="inlineStr">
+        <is>
+          <t>748</t>
+        </is>
+      </c>
+      <c r="AR22" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="AS22" t="inlineStr">
+        <is>
+          <t>748</t>
+        </is>
+      </c>
+      <c r="AT22" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="AU22" t="inlineStr">
+        <is>
+          <t>748</t>
+        </is>
+      </c>
+      <c r="AV22" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="AW22" t="inlineStr">
+        <is>
+          <t>748</t>
+        </is>
+      </c>
+      <c r="AX22" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="AY22" t="inlineStr">
+        <is>
+          <t>748</t>
+        </is>
+      </c>
+      <c r="AZ22" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="BA22" t="inlineStr">
+        <is>
+          <t>748</t>
+        </is>
+      </c>
+      <c r="BB22" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="BC22" t="inlineStr">
+        <is>
+          <t>748</t>
+        </is>
+      </c>
+      <c r="BD22" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="BE22" t="inlineStr">
+        <is>
+          <t>748</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -4832,6 +6740,96 @@
       <c r="AM23" t="inlineStr">
         <is>
           <t>698</t>
+        </is>
+      </c>
+      <c r="AN23" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="AO23" t="inlineStr">
+        <is>
+          <t>698</t>
+        </is>
+      </c>
+      <c r="AP23" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="AQ23" t="inlineStr">
+        <is>
+          <t>748</t>
+        </is>
+      </c>
+      <c r="AR23" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="AS23" t="inlineStr">
+        <is>
+          <t>748</t>
+        </is>
+      </c>
+      <c r="AT23" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="AU23" t="inlineStr">
+        <is>
+          <t>748</t>
+        </is>
+      </c>
+      <c r="AV23" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="AW23" t="inlineStr">
+        <is>
+          <t>748</t>
+        </is>
+      </c>
+      <c r="AX23" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="AY23" t="inlineStr">
+        <is>
+          <t>748</t>
+        </is>
+      </c>
+      <c r="AZ23" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="BA23" t="inlineStr">
+        <is>
+          <t>748</t>
+        </is>
+      </c>
+      <c r="BB23" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="BC23" t="inlineStr">
+        <is>
+          <t>748</t>
+        </is>
+      </c>
+      <c r="BD23" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="BE23" t="inlineStr">
+        <is>
+          <t>748</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Updated XPaths for websites and scraper results.
</commit_message>
<xml_diff>
--- a/price_extractor.xlsx
+++ b/price_extractor.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BE23"/>
+  <dimension ref="A1:CM23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -714,6 +714,176 @@
           <t>Price_2025-03-04 17:48</t>
         </is>
       </c>
+      <c r="BF1" s="1" t="inlineStr">
+        <is>
+          <t>Product Name_2025-03-05 03:05</t>
+        </is>
+      </c>
+      <c r="BG1" s="1" t="inlineStr">
+        <is>
+          <t>Price_2025-03-05 03:05</t>
+        </is>
+      </c>
+      <c r="BH1" s="1" t="inlineStr">
+        <is>
+          <t>Product Name_2025-03-06 03:05</t>
+        </is>
+      </c>
+      <c r="BI1" s="1" t="inlineStr">
+        <is>
+          <t>Price_2025-03-06 03:05</t>
+        </is>
+      </c>
+      <c r="BJ1" s="1" t="inlineStr">
+        <is>
+          <t>Product Name_2025-03-07 03:04</t>
+        </is>
+      </c>
+      <c r="BK1" s="1" t="inlineStr">
+        <is>
+          <t>Price_2025-03-07 03:04</t>
+        </is>
+      </c>
+      <c r="BL1" s="1" t="inlineStr">
+        <is>
+          <t>Product Name_2025-03-08 03:04</t>
+        </is>
+      </c>
+      <c r="BM1" s="1" t="inlineStr">
+        <is>
+          <t>Price_2025-03-08 03:04</t>
+        </is>
+      </c>
+      <c r="BN1" s="1" t="inlineStr">
+        <is>
+          <t>Product Name_2025-03-09 03:04</t>
+        </is>
+      </c>
+      <c r="BO1" s="1" t="inlineStr">
+        <is>
+          <t>Price_2025-03-09 03:04</t>
+        </is>
+      </c>
+      <c r="BP1" s="1" t="inlineStr">
+        <is>
+          <t>Product Name_2025-03-10 03:05</t>
+        </is>
+      </c>
+      <c r="BQ1" s="1" t="inlineStr">
+        <is>
+          <t>Price_2025-03-10 03:05</t>
+        </is>
+      </c>
+      <c r="BR1" s="1" t="inlineStr">
+        <is>
+          <t>Product Name_2025-03-11 03:04</t>
+        </is>
+      </c>
+      <c r="BS1" s="1" t="inlineStr">
+        <is>
+          <t>Price_2025-03-11 03:04</t>
+        </is>
+      </c>
+      <c r="BT1" s="1" t="inlineStr">
+        <is>
+          <t>Product Name_2025-03-12 03:05</t>
+        </is>
+      </c>
+      <c r="BU1" s="1" t="inlineStr">
+        <is>
+          <t>Price_2025-03-12 03:05</t>
+        </is>
+      </c>
+      <c r="BV1" s="1" t="inlineStr">
+        <is>
+          <t>Product Name_2025-03-13 03:05</t>
+        </is>
+      </c>
+      <c r="BW1" s="1" t="inlineStr">
+        <is>
+          <t>Price_2025-03-13 03:05</t>
+        </is>
+      </c>
+      <c r="BX1" s="1" t="inlineStr">
+        <is>
+          <t>Product Name_2025-03-14 03:04</t>
+        </is>
+      </c>
+      <c r="BY1" s="1" t="inlineStr">
+        <is>
+          <t>Price_2025-03-14 03:04</t>
+        </is>
+      </c>
+      <c r="BZ1" s="1" t="inlineStr">
+        <is>
+          <t>Product Name_2025-03-15 03:05</t>
+        </is>
+      </c>
+      <c r="CA1" s="1" t="inlineStr">
+        <is>
+          <t>Price_2025-03-15 03:05</t>
+        </is>
+      </c>
+      <c r="CB1" s="1" t="inlineStr">
+        <is>
+          <t>Product Name_2025-03-16 03:04</t>
+        </is>
+      </c>
+      <c r="CC1" s="1" t="inlineStr">
+        <is>
+          <t>Price_2025-03-16 03:04</t>
+        </is>
+      </c>
+      <c r="CD1" s="1" t="inlineStr">
+        <is>
+          <t>Product Name_2025-03-17 03:05</t>
+        </is>
+      </c>
+      <c r="CE1" s="1" t="inlineStr">
+        <is>
+          <t>Price_2025-03-17 03:05</t>
+        </is>
+      </c>
+      <c r="CF1" s="1" t="inlineStr">
+        <is>
+          <t>Product Name_2025-03-18 03:04</t>
+        </is>
+      </c>
+      <c r="CG1" s="1" t="inlineStr">
+        <is>
+          <t>Price_2025-03-18 03:04</t>
+        </is>
+      </c>
+      <c r="CH1" s="1" t="inlineStr">
+        <is>
+          <t>Product Name_2025-03-19 03:04</t>
+        </is>
+      </c>
+      <c r="CI1" s="1" t="inlineStr">
+        <is>
+          <t>Price_2025-03-19 03:04</t>
+        </is>
+      </c>
+      <c r="CJ1" s="1" t="inlineStr">
+        <is>
+          <t>Product Name_2025-03-20 03:05</t>
+        </is>
+      </c>
+      <c r="CK1" s="1" t="inlineStr">
+        <is>
+          <t>Price_2025-03-20 03:05</t>
+        </is>
+      </c>
+      <c r="CL1" s="1" t="inlineStr">
+        <is>
+          <t>Product Name_2025-03-21 03:05</t>
+        </is>
+      </c>
+      <c r="CM1" s="1" t="inlineStr">
+        <is>
+          <t>Price_2025-03-21 03:05</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1001,6 +1171,176 @@
           <t>2.899</t>
         </is>
       </c>
+      <c r="BF2" t="inlineStr">
+        <is>
+          <t>UNLEADED 87 (10% ETH)</t>
+        </is>
+      </c>
+      <c r="BG2" t="inlineStr">
+        <is>
+          <t>2.899</t>
+        </is>
+      </c>
+      <c r="BH2" t="inlineStr">
+        <is>
+          <t>UNLEADED 87 (10% ETH)</t>
+        </is>
+      </c>
+      <c r="BI2" t="inlineStr">
+        <is>
+          <t>2.849</t>
+        </is>
+      </c>
+      <c r="BJ2" t="inlineStr">
+        <is>
+          <t>UNLEADED 87 (10% ETH)</t>
+        </is>
+      </c>
+      <c r="BK2" t="inlineStr">
+        <is>
+          <t>2.849</t>
+        </is>
+      </c>
+      <c r="BL2" t="inlineStr">
+        <is>
+          <t>UNLEADED 87 (10% ETH)</t>
+        </is>
+      </c>
+      <c r="BM2" t="inlineStr">
+        <is>
+          <t>2.799</t>
+        </is>
+      </c>
+      <c r="BN2" t="inlineStr">
+        <is>
+          <t>UNLEADED 87 (10% ETH)</t>
+        </is>
+      </c>
+      <c r="BO2" t="inlineStr">
+        <is>
+          <t>2.799</t>
+        </is>
+      </c>
+      <c r="BP2" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="BQ2" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="BR2" t="inlineStr">
+        <is>
+          <t>UNLEADED 87 (10% ETH)</t>
+        </is>
+      </c>
+      <c r="BS2" t="inlineStr">
+        <is>
+          <t>2.749</t>
+        </is>
+      </c>
+      <c r="BT2" t="inlineStr">
+        <is>
+          <t>UNLEADED 87 (10% ETH)</t>
+        </is>
+      </c>
+      <c r="BU2" t="inlineStr">
+        <is>
+          <t>2.699</t>
+        </is>
+      </c>
+      <c r="BV2" t="inlineStr">
+        <is>
+          <t>UNLEADED 87 (10% ETH)</t>
+        </is>
+      </c>
+      <c r="BW2" t="inlineStr">
+        <is>
+          <t>2.649</t>
+        </is>
+      </c>
+      <c r="BX2" t="inlineStr">
+        <is>
+          <t>UNLEADED 87 (10% ETH)</t>
+        </is>
+      </c>
+      <c r="BY2" t="inlineStr">
+        <is>
+          <t>2.599</t>
+        </is>
+      </c>
+      <c r="BZ2" t="inlineStr">
+        <is>
+          <t>UNLEADED 87 (10% ETH)</t>
+        </is>
+      </c>
+      <c r="CA2" t="inlineStr">
+        <is>
+          <t>2.599</t>
+        </is>
+      </c>
+      <c r="CB2" t="inlineStr">
+        <is>
+          <t>UNLEADED 87 (10% ETH)</t>
+        </is>
+      </c>
+      <c r="CC2" t="inlineStr">
+        <is>
+          <t>2.599</t>
+        </is>
+      </c>
+      <c r="CD2" t="inlineStr">
+        <is>
+          <t>UNLEADED 87 (10% ETH)</t>
+        </is>
+      </c>
+      <c r="CE2" t="inlineStr">
+        <is>
+          <t>2.599</t>
+        </is>
+      </c>
+      <c r="CF2" t="inlineStr">
+        <is>
+          <t>UNLEADED 87 (10% ETH)</t>
+        </is>
+      </c>
+      <c r="CG2" t="inlineStr">
+        <is>
+          <t>2.899</t>
+        </is>
+      </c>
+      <c r="CH2" t="inlineStr">
+        <is>
+          <t>UNLEADED 87 (10% ETH)</t>
+        </is>
+      </c>
+      <c r="CI2" t="inlineStr">
+        <is>
+          <t>2.899</t>
+        </is>
+      </c>
+      <c r="CJ2" t="inlineStr">
+        <is>
+          <t>UNLEADED 87 (10% ETH)</t>
+        </is>
+      </c>
+      <c r="CK2" t="inlineStr">
+        <is>
+          <t>2.899</t>
+        </is>
+      </c>
+      <c r="CL2" t="inlineStr">
+        <is>
+          <t>UNLEADED 87 (10% ETH)</t>
+        </is>
+      </c>
+      <c r="CM2" t="inlineStr">
+        <is>
+          <t>2.899</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1288,6 +1628,176 @@
           <t>$2.72</t>
         </is>
       </c>
+      <c r="BF3" t="inlineStr">
+        <is>
+          <t>That's Smart! Fat Free Skim Milk</t>
+        </is>
+      </c>
+      <c r="BG3" t="inlineStr">
+        <is>
+          <t>$2.72</t>
+        </is>
+      </c>
+      <c r="BH3" t="inlineStr">
+        <is>
+          <t>That's Smart! Fat Free Skim Milk</t>
+        </is>
+      </c>
+      <c r="BI3" t="inlineStr">
+        <is>
+          <t>$2.72</t>
+        </is>
+      </c>
+      <c r="BJ3" t="inlineStr">
+        <is>
+          <t>That's Smart! Fat Free Skim Milk</t>
+        </is>
+      </c>
+      <c r="BK3" t="inlineStr">
+        <is>
+          <t>$2.72</t>
+        </is>
+      </c>
+      <c r="BL3" t="inlineStr">
+        <is>
+          <t>That's Smart! Fat Free Skim Milk</t>
+        </is>
+      </c>
+      <c r="BM3" t="inlineStr">
+        <is>
+          <t>$2.72</t>
+        </is>
+      </c>
+      <c r="BN3" t="inlineStr">
+        <is>
+          <t>That's Smart! Fat Free Skim Milk</t>
+        </is>
+      </c>
+      <c r="BO3" t="inlineStr">
+        <is>
+          <t>$2.72</t>
+        </is>
+      </c>
+      <c r="BP3" t="inlineStr">
+        <is>
+          <t>That's Smart! Fat Free Skim Milk</t>
+        </is>
+      </c>
+      <c r="BQ3" t="inlineStr">
+        <is>
+          <t>$2.72</t>
+        </is>
+      </c>
+      <c r="BR3" t="inlineStr">
+        <is>
+          <t>That's Smart! Fat Free Skim Milk</t>
+        </is>
+      </c>
+      <c r="BS3" t="inlineStr">
+        <is>
+          <t>$2.72</t>
+        </is>
+      </c>
+      <c r="BT3" t="inlineStr">
+        <is>
+          <t>That's Smart! Fat Free Skim Milk</t>
+        </is>
+      </c>
+      <c r="BU3" t="inlineStr">
+        <is>
+          <t>$2.72</t>
+        </is>
+      </c>
+      <c r="BV3" t="inlineStr">
+        <is>
+          <t>That's Smart! Fat Free Skim Milk</t>
+        </is>
+      </c>
+      <c r="BW3" t="inlineStr">
+        <is>
+          <t>$2.72</t>
+        </is>
+      </c>
+      <c r="BX3" t="inlineStr">
+        <is>
+          <t>That's Smart! Fat Free Skim Milk</t>
+        </is>
+      </c>
+      <c r="BY3" t="inlineStr">
+        <is>
+          <t>$2.72</t>
+        </is>
+      </c>
+      <c r="BZ3" t="inlineStr">
+        <is>
+          <t>That's Smart! Fat Free Skim Milk</t>
+        </is>
+      </c>
+      <c r="CA3" t="inlineStr">
+        <is>
+          <t>$2.72</t>
+        </is>
+      </c>
+      <c r="CB3" t="inlineStr">
+        <is>
+          <t>That's Smart! Fat Free Skim Milk</t>
+        </is>
+      </c>
+      <c r="CC3" t="inlineStr">
+        <is>
+          <t>$2.72</t>
+        </is>
+      </c>
+      <c r="CD3" t="inlineStr">
+        <is>
+          <t>That's Smart! Fat Free Skim Milk</t>
+        </is>
+      </c>
+      <c r="CE3" t="inlineStr">
+        <is>
+          <t>$2.72</t>
+        </is>
+      </c>
+      <c r="CF3" t="inlineStr">
+        <is>
+          <t>That's Smart! Fat Free Skim Milk</t>
+        </is>
+      </c>
+      <c r="CG3" t="inlineStr">
+        <is>
+          <t>$2.72</t>
+        </is>
+      </c>
+      <c r="CH3" t="inlineStr">
+        <is>
+          <t>That's Smart! Fat Free Skim Milk</t>
+        </is>
+      </c>
+      <c r="CI3" t="inlineStr">
+        <is>
+          <t>$2.72</t>
+        </is>
+      </c>
+      <c r="CJ3" t="inlineStr">
+        <is>
+          <t>That's Smart! Fat Free Skim Milk</t>
+        </is>
+      </c>
+      <c r="CK3" t="inlineStr">
+        <is>
+          <t>$2.72</t>
+        </is>
+      </c>
+      <c r="CL3" t="inlineStr">
+        <is>
+          <t>That's Smart! Fat Free Skim Milk</t>
+        </is>
+      </c>
+      <c r="CM3" t="inlineStr">
+        <is>
+          <t>$2.72</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1575,6 +2085,176 @@
           <t>38¢ ea.</t>
         </is>
       </c>
+      <c r="BF4" t="inlineStr">
+        <is>
+          <t>Roma Tomatoes</t>
+        </is>
+      </c>
+      <c r="BG4" t="inlineStr">
+        <is>
+          <t>38¢ ea.</t>
+        </is>
+      </c>
+      <c r="BH4" t="inlineStr">
+        <is>
+          <t>Roma Tomatoes</t>
+        </is>
+      </c>
+      <c r="BI4" t="inlineStr">
+        <is>
+          <t>38¢ ea.</t>
+        </is>
+      </c>
+      <c r="BJ4" t="inlineStr">
+        <is>
+          <t>Roma Tomatoes</t>
+        </is>
+      </c>
+      <c r="BK4" t="inlineStr">
+        <is>
+          <t>38¢ ea.</t>
+        </is>
+      </c>
+      <c r="BL4" t="inlineStr">
+        <is>
+          <t>Roma Tomatoes</t>
+        </is>
+      </c>
+      <c r="BM4" t="inlineStr">
+        <is>
+          <t>38¢ ea.</t>
+        </is>
+      </c>
+      <c r="BN4" t="inlineStr">
+        <is>
+          <t>Roma Tomatoes</t>
+        </is>
+      </c>
+      <c r="BO4" t="inlineStr">
+        <is>
+          <t>38¢ ea.</t>
+        </is>
+      </c>
+      <c r="BP4" t="inlineStr">
+        <is>
+          <t>Roma Tomatoes</t>
+        </is>
+      </c>
+      <c r="BQ4" t="inlineStr">
+        <is>
+          <t>32¢ ea.</t>
+        </is>
+      </c>
+      <c r="BR4" t="inlineStr">
+        <is>
+          <t>Roma Tomatoes</t>
+        </is>
+      </c>
+      <c r="BS4" t="inlineStr">
+        <is>
+          <t>32¢ ea.</t>
+        </is>
+      </c>
+      <c r="BT4" t="inlineStr">
+        <is>
+          <t>Roma Tomatoes</t>
+        </is>
+      </c>
+      <c r="BU4" t="inlineStr">
+        <is>
+          <t>32¢ ea.</t>
+        </is>
+      </c>
+      <c r="BV4" t="inlineStr">
+        <is>
+          <t>Roma Tomatoes</t>
+        </is>
+      </c>
+      <c r="BW4" t="inlineStr">
+        <is>
+          <t>32¢ ea.</t>
+        </is>
+      </c>
+      <c r="BX4" t="inlineStr">
+        <is>
+          <t>Roma Tomatoes</t>
+        </is>
+      </c>
+      <c r="BY4" t="inlineStr">
+        <is>
+          <t>32¢ ea.</t>
+        </is>
+      </c>
+      <c r="BZ4" t="inlineStr">
+        <is>
+          <t>Roma Tomatoes</t>
+        </is>
+      </c>
+      <c r="CA4" t="inlineStr">
+        <is>
+          <t>32¢ ea.</t>
+        </is>
+      </c>
+      <c r="CB4" t="inlineStr">
+        <is>
+          <t>Roma Tomatoes</t>
+        </is>
+      </c>
+      <c r="CC4" t="inlineStr">
+        <is>
+          <t>32¢ ea.</t>
+        </is>
+      </c>
+      <c r="CD4" t="inlineStr">
+        <is>
+          <t>Roma Tomatoes</t>
+        </is>
+      </c>
+      <c r="CE4" t="inlineStr">
+        <is>
+          <t>38¢ ea.</t>
+        </is>
+      </c>
+      <c r="CF4" t="inlineStr">
+        <is>
+          <t>Roma Tomatoes</t>
+        </is>
+      </c>
+      <c r="CG4" t="inlineStr">
+        <is>
+          <t>38¢ ea.</t>
+        </is>
+      </c>
+      <c r="CH4" t="inlineStr">
+        <is>
+          <t>Roma Tomatoes</t>
+        </is>
+      </c>
+      <c r="CI4" t="inlineStr">
+        <is>
+          <t>38¢ ea.</t>
+        </is>
+      </c>
+      <c r="CJ4" t="inlineStr">
+        <is>
+          <t>Roma Tomatoes</t>
+        </is>
+      </c>
+      <c r="CK4" t="inlineStr">
+        <is>
+          <t>38¢ ea.</t>
+        </is>
+      </c>
+      <c r="CL4" t="inlineStr">
+        <is>
+          <t>Roma Tomatoes</t>
+        </is>
+      </c>
+      <c r="CM4" t="inlineStr">
+        <is>
+          <t>38¢ ea.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1862,6 +2542,176 @@
           <t>$4.97</t>
         </is>
       </c>
+      <c r="BF5" t="inlineStr">
+        <is>
+          <t>Quaker Cap'n Crunch Regular Cereal</t>
+        </is>
+      </c>
+      <c r="BG5" t="inlineStr">
+        <is>
+          <t>$4.97</t>
+        </is>
+      </c>
+      <c r="BH5" t="inlineStr">
+        <is>
+          <t>Quaker Cap'n Crunch Regular Cereal</t>
+        </is>
+      </c>
+      <c r="BI5" t="inlineStr">
+        <is>
+          <t>$4.97</t>
+        </is>
+      </c>
+      <c r="BJ5" t="inlineStr">
+        <is>
+          <t>Quaker Cap'n Crunch Regular Cereal</t>
+        </is>
+      </c>
+      <c r="BK5" t="inlineStr">
+        <is>
+          <t>$4.97</t>
+        </is>
+      </c>
+      <c r="BL5" t="inlineStr">
+        <is>
+          <t>Quaker Cap'n Crunch Regular Cereal</t>
+        </is>
+      </c>
+      <c r="BM5" t="inlineStr">
+        <is>
+          <t>$4.97</t>
+        </is>
+      </c>
+      <c r="BN5" t="inlineStr">
+        <is>
+          <t>Quaker Cap'n Crunch Regular Cereal</t>
+        </is>
+      </c>
+      <c r="BO5" t="inlineStr">
+        <is>
+          <t>$4.97</t>
+        </is>
+      </c>
+      <c r="BP5" t="inlineStr">
+        <is>
+          <t>Quaker Cap'n Crunch Regular Cereal</t>
+        </is>
+      </c>
+      <c r="BQ5" t="inlineStr">
+        <is>
+          <t>$4.97</t>
+        </is>
+      </c>
+      <c r="BR5" t="inlineStr">
+        <is>
+          <t>Quaker Cap'n Crunch Regular Cereal</t>
+        </is>
+      </c>
+      <c r="BS5" t="inlineStr">
+        <is>
+          <t>$4.97</t>
+        </is>
+      </c>
+      <c r="BT5" t="inlineStr">
+        <is>
+          <t>Quaker Cap'n Crunch Regular Cereal</t>
+        </is>
+      </c>
+      <c r="BU5" t="inlineStr">
+        <is>
+          <t>$4.97</t>
+        </is>
+      </c>
+      <c r="BV5" t="inlineStr">
+        <is>
+          <t>Quaker Cap'n Crunch Regular Cereal</t>
+        </is>
+      </c>
+      <c r="BW5" t="inlineStr">
+        <is>
+          <t>$4.97</t>
+        </is>
+      </c>
+      <c r="BX5" t="inlineStr">
+        <is>
+          <t>Quaker Cap'n Crunch Regular Cereal</t>
+        </is>
+      </c>
+      <c r="BY5" t="inlineStr">
+        <is>
+          <t>$4.97</t>
+        </is>
+      </c>
+      <c r="BZ5" t="inlineStr">
+        <is>
+          <t>Quaker Cap'n Crunch Regular Cereal</t>
+        </is>
+      </c>
+      <c r="CA5" t="inlineStr">
+        <is>
+          <t>$4.97</t>
+        </is>
+      </c>
+      <c r="CB5" t="inlineStr">
+        <is>
+          <t>Quaker Cap'n Crunch Regular Cereal</t>
+        </is>
+      </c>
+      <c r="CC5" t="inlineStr">
+        <is>
+          <t>$4.97</t>
+        </is>
+      </c>
+      <c r="CD5" t="inlineStr">
+        <is>
+          <t>Quaker Cap'n Crunch Regular Cereal</t>
+        </is>
+      </c>
+      <c r="CE5" t="inlineStr">
+        <is>
+          <t>$4.97</t>
+        </is>
+      </c>
+      <c r="CF5" t="inlineStr">
+        <is>
+          <t>Quaker Cap'n Crunch Regular Cereal</t>
+        </is>
+      </c>
+      <c r="CG5" t="inlineStr">
+        <is>
+          <t>$4.97</t>
+        </is>
+      </c>
+      <c r="CH5" t="inlineStr">
+        <is>
+          <t>Quaker Cap'n Crunch Regular Cereal</t>
+        </is>
+      </c>
+      <c r="CI5" t="inlineStr">
+        <is>
+          <t>$4.97</t>
+        </is>
+      </c>
+      <c r="CJ5" t="inlineStr">
+        <is>
+          <t>Quaker Cap'n Crunch Regular Cereal</t>
+        </is>
+      </c>
+      <c r="CK5" t="inlineStr">
+        <is>
+          <t>$4.97</t>
+        </is>
+      </c>
+      <c r="CL5" t="inlineStr">
+        <is>
+          <t>Quaker Cap'n Crunch Regular Cereal</t>
+        </is>
+      </c>
+      <c r="CM5" t="inlineStr">
+        <is>
+          <t>$4.97</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -2149,6 +2999,176 @@
           <t>$3.99</t>
         </is>
       </c>
+      <c r="BF6" t="inlineStr">
+        <is>
+          <t>Sara Lee Artesano Brioche Buns, 8 count</t>
+        </is>
+      </c>
+      <c r="BG6" t="inlineStr">
+        <is>
+          <t>$3.99</t>
+        </is>
+      </c>
+      <c r="BH6" t="inlineStr">
+        <is>
+          <t>Sara Lee Artesano Brioche Buns, 8 count</t>
+        </is>
+      </c>
+      <c r="BI6" t="inlineStr">
+        <is>
+          <t>$3.99</t>
+        </is>
+      </c>
+      <c r="BJ6" t="inlineStr">
+        <is>
+          <t>Sara Lee Artesano Brioche Buns, 8 count</t>
+        </is>
+      </c>
+      <c r="BK6" t="inlineStr">
+        <is>
+          <t>$3.99</t>
+        </is>
+      </c>
+      <c r="BL6" t="inlineStr">
+        <is>
+          <t>Sara Lee Artesano Brioche Buns, 8 count</t>
+        </is>
+      </c>
+      <c r="BM6" t="inlineStr">
+        <is>
+          <t>$3.99</t>
+        </is>
+      </c>
+      <c r="BN6" t="inlineStr">
+        <is>
+          <t>Sara Lee Artesano Brioche Buns, 8 count</t>
+        </is>
+      </c>
+      <c r="BO6" t="inlineStr">
+        <is>
+          <t>$3.99</t>
+        </is>
+      </c>
+      <c r="BP6" t="inlineStr">
+        <is>
+          <t>Sara Lee Artesano Brioche Buns, 8 count</t>
+        </is>
+      </c>
+      <c r="BQ6" t="inlineStr">
+        <is>
+          <t>$3.99</t>
+        </is>
+      </c>
+      <c r="BR6" t="inlineStr">
+        <is>
+          <t>Sara Lee Artesano Brioche Buns, 8 count</t>
+        </is>
+      </c>
+      <c r="BS6" t="inlineStr">
+        <is>
+          <t>$3.99</t>
+        </is>
+      </c>
+      <c r="BT6" t="inlineStr">
+        <is>
+          <t>Sara Lee Artesano Brioche Buns, 8 count</t>
+        </is>
+      </c>
+      <c r="BU6" t="inlineStr">
+        <is>
+          <t>$3.99</t>
+        </is>
+      </c>
+      <c r="BV6" t="inlineStr">
+        <is>
+          <t>Sara Lee Artesano Brioche Buns, 8 count</t>
+        </is>
+      </c>
+      <c r="BW6" t="inlineStr">
+        <is>
+          <t>$3.99</t>
+        </is>
+      </c>
+      <c r="BX6" t="inlineStr">
+        <is>
+          <t>Sara Lee Artesano Brioche Buns, 8 count</t>
+        </is>
+      </c>
+      <c r="BY6" t="inlineStr">
+        <is>
+          <t>$3.99</t>
+        </is>
+      </c>
+      <c r="BZ6" t="inlineStr">
+        <is>
+          <t>Sara Lee Artesano Brioche Buns, 8 count</t>
+        </is>
+      </c>
+      <c r="CA6" t="inlineStr">
+        <is>
+          <t>$3.99</t>
+        </is>
+      </c>
+      <c r="CB6" t="inlineStr">
+        <is>
+          <t>Sara Lee Artesano Brioche Buns, 8 count</t>
+        </is>
+      </c>
+      <c r="CC6" t="inlineStr">
+        <is>
+          <t>$3.99</t>
+        </is>
+      </c>
+      <c r="CD6" t="inlineStr">
+        <is>
+          <t>Sara Lee Artesano Brioche Buns, 8 count</t>
+        </is>
+      </c>
+      <c r="CE6" t="inlineStr">
+        <is>
+          <t>$3.99</t>
+        </is>
+      </c>
+      <c r="CF6" t="inlineStr">
+        <is>
+          <t>Sara Lee Artesano Brioche Buns, 8 count</t>
+        </is>
+      </c>
+      <c r="CG6" t="inlineStr">
+        <is>
+          <t>$3.99</t>
+        </is>
+      </c>
+      <c r="CH6" t="inlineStr">
+        <is>
+          <t>Sara Lee Artesano Brioche Buns, 8 count</t>
+        </is>
+      </c>
+      <c r="CI6" t="inlineStr">
+        <is>
+          <t>$3.99</t>
+        </is>
+      </c>
+      <c r="CJ6" t="inlineStr">
+        <is>
+          <t>Sara Lee Artesano Brioche Buns, 8 count</t>
+        </is>
+      </c>
+      <c r="CK6" t="inlineStr">
+        <is>
+          <t>$3.99</t>
+        </is>
+      </c>
+      <c r="CL6" t="inlineStr">
+        <is>
+          <t>Sara Lee Artesano Brioche Buns, 8 count</t>
+        </is>
+      </c>
+      <c r="CM6" t="inlineStr">
+        <is>
+          <t>$3.99</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -2436,6 +3456,176 @@
           <t>$3.65</t>
         </is>
       </c>
+      <c r="BF7" t="inlineStr">
+        <is>
+          <t>That's Smart! Mayonnaise</t>
+        </is>
+      </c>
+      <c r="BG7" t="inlineStr">
+        <is>
+          <t>$3.65</t>
+        </is>
+      </c>
+      <c r="BH7" t="inlineStr">
+        <is>
+          <t>That's Smart! Mayonnaise</t>
+        </is>
+      </c>
+      <c r="BI7" t="inlineStr">
+        <is>
+          <t>$3.65</t>
+        </is>
+      </c>
+      <c r="BJ7" t="inlineStr">
+        <is>
+          <t>That's Smart! Mayonnaise</t>
+        </is>
+      </c>
+      <c r="BK7" t="inlineStr">
+        <is>
+          <t>$3.65</t>
+        </is>
+      </c>
+      <c r="BL7" t="inlineStr">
+        <is>
+          <t>That's Smart! Mayonnaise</t>
+        </is>
+      </c>
+      <c r="BM7" t="inlineStr">
+        <is>
+          <t>$3.65</t>
+        </is>
+      </c>
+      <c r="BN7" t="inlineStr">
+        <is>
+          <t>That's Smart! Mayonnaise</t>
+        </is>
+      </c>
+      <c r="BO7" t="inlineStr">
+        <is>
+          <t>$3.65</t>
+        </is>
+      </c>
+      <c r="BP7" t="inlineStr">
+        <is>
+          <t>That's Smart! Mayonnaise</t>
+        </is>
+      </c>
+      <c r="BQ7" t="inlineStr">
+        <is>
+          <t>$3.65</t>
+        </is>
+      </c>
+      <c r="BR7" t="inlineStr">
+        <is>
+          <t>That's Smart! Mayonnaise</t>
+        </is>
+      </c>
+      <c r="BS7" t="inlineStr">
+        <is>
+          <t>$3.65</t>
+        </is>
+      </c>
+      <c r="BT7" t="inlineStr">
+        <is>
+          <t>That's Smart! Mayonnaise</t>
+        </is>
+      </c>
+      <c r="BU7" t="inlineStr">
+        <is>
+          <t>$3.65</t>
+        </is>
+      </c>
+      <c r="BV7" t="inlineStr">
+        <is>
+          <t>That's Smart! Mayonnaise</t>
+        </is>
+      </c>
+      <c r="BW7" t="inlineStr">
+        <is>
+          <t>$3.65</t>
+        </is>
+      </c>
+      <c r="BX7" t="inlineStr">
+        <is>
+          <t>That's Smart! Mayonnaise</t>
+        </is>
+      </c>
+      <c r="BY7" t="inlineStr">
+        <is>
+          <t>$3.65</t>
+        </is>
+      </c>
+      <c r="BZ7" t="inlineStr">
+        <is>
+          <t>That's Smart! Mayonnaise</t>
+        </is>
+      </c>
+      <c r="CA7" t="inlineStr">
+        <is>
+          <t>$3.65</t>
+        </is>
+      </c>
+      <c r="CB7" t="inlineStr">
+        <is>
+          <t>That's Smart! Mayonnaise</t>
+        </is>
+      </c>
+      <c r="CC7" t="inlineStr">
+        <is>
+          <t>$3.65</t>
+        </is>
+      </c>
+      <c r="CD7" t="inlineStr">
+        <is>
+          <t>That's Smart! Mayonnaise</t>
+        </is>
+      </c>
+      <c r="CE7" t="inlineStr">
+        <is>
+          <t>$3.65</t>
+        </is>
+      </c>
+      <c r="CF7" t="inlineStr">
+        <is>
+          <t>That's Smart! Mayonnaise</t>
+        </is>
+      </c>
+      <c r="CG7" t="inlineStr">
+        <is>
+          <t>$3.65</t>
+        </is>
+      </c>
+      <c r="CH7" t="inlineStr">
+        <is>
+          <t>That's Smart! Mayonnaise</t>
+        </is>
+      </c>
+      <c r="CI7" t="inlineStr">
+        <is>
+          <t>$3.65</t>
+        </is>
+      </c>
+      <c r="CJ7" t="inlineStr">
+        <is>
+          <t>That's Smart! Mayonnaise</t>
+        </is>
+      </c>
+      <c r="CK7" t="inlineStr">
+        <is>
+          <t>$3.65</t>
+        </is>
+      </c>
+      <c r="CL7" t="inlineStr">
+        <is>
+          <t>That's Smart! Mayonnaise</t>
+        </is>
+      </c>
+      <c r="CM7" t="inlineStr">
+        <is>
+          <t>$3.65</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -2723,6 +3913,176 @@
           <t>$1.99</t>
         </is>
       </c>
+      <c r="BF8" t="inlineStr">
+        <is>
+          <t>Hy-Vee Light Bartlett Pear Halves In Pear Juice From Concentrate</t>
+        </is>
+      </c>
+      <c r="BG8" t="inlineStr">
+        <is>
+          <t>$1.99</t>
+        </is>
+      </c>
+      <c r="BH8" t="inlineStr">
+        <is>
+          <t>Hy-Vee Light Bartlett Pear Halves In Pear Juice From Concentrate</t>
+        </is>
+      </c>
+      <c r="BI8" t="inlineStr">
+        <is>
+          <t>$1.99</t>
+        </is>
+      </c>
+      <c r="BJ8" t="inlineStr">
+        <is>
+          <t>Hy-Vee Light Bartlett Pear Halves In Pear Juice From Concentrate</t>
+        </is>
+      </c>
+      <c r="BK8" t="inlineStr">
+        <is>
+          <t>$1.99</t>
+        </is>
+      </c>
+      <c r="BL8" t="inlineStr">
+        <is>
+          <t>Hy-Vee Light Bartlett Pear Halves In Pear Juice From Concentrate</t>
+        </is>
+      </c>
+      <c r="BM8" t="inlineStr">
+        <is>
+          <t>$1.99</t>
+        </is>
+      </c>
+      <c r="BN8" t="inlineStr">
+        <is>
+          <t>Hy-Vee Light Bartlett Pear Halves In Pear Juice From Concentrate</t>
+        </is>
+      </c>
+      <c r="BO8" t="inlineStr">
+        <is>
+          <t>$1.99</t>
+        </is>
+      </c>
+      <c r="BP8" t="inlineStr">
+        <is>
+          <t>Hy-Vee Light Bartlett Pear Halves In Pear Juice From Concentrate</t>
+        </is>
+      </c>
+      <c r="BQ8" t="inlineStr">
+        <is>
+          <t>$1.99</t>
+        </is>
+      </c>
+      <c r="BR8" t="inlineStr">
+        <is>
+          <t>Hy-Vee Light Bartlett Pear Halves In Pear Juice From Concentrate</t>
+        </is>
+      </c>
+      <c r="BS8" t="inlineStr">
+        <is>
+          <t>$1.99</t>
+        </is>
+      </c>
+      <c r="BT8" t="inlineStr">
+        <is>
+          <t>Hy-Vee Light Bartlett Pear Halves In Pear Juice From Concentrate</t>
+        </is>
+      </c>
+      <c r="BU8" t="inlineStr">
+        <is>
+          <t>$1.99</t>
+        </is>
+      </c>
+      <c r="BV8" t="inlineStr">
+        <is>
+          <t>Hy-Vee Light Bartlett Pear Halves In Pear Juice From Concentrate</t>
+        </is>
+      </c>
+      <c r="BW8" t="inlineStr">
+        <is>
+          <t>$1.99</t>
+        </is>
+      </c>
+      <c r="BX8" t="inlineStr">
+        <is>
+          <t>Hy-Vee Light Bartlett Pear Halves In Pear Juice From Concentrate</t>
+        </is>
+      </c>
+      <c r="BY8" t="inlineStr">
+        <is>
+          <t>$1.99</t>
+        </is>
+      </c>
+      <c r="BZ8" t="inlineStr">
+        <is>
+          <t>Hy-Vee Light Bartlett Pear Halves In Pear Juice From Concentrate</t>
+        </is>
+      </c>
+      <c r="CA8" t="inlineStr">
+        <is>
+          <t>$1.99</t>
+        </is>
+      </c>
+      <c r="CB8" t="inlineStr">
+        <is>
+          <t>Hy-Vee Light Bartlett Pear Halves In Pear Juice From Concentrate</t>
+        </is>
+      </c>
+      <c r="CC8" t="inlineStr">
+        <is>
+          <t>$1.99</t>
+        </is>
+      </c>
+      <c r="CD8" t="inlineStr">
+        <is>
+          <t>Hy-Vee Light Bartlett Pear Halves In Pear Juice From Concentrate</t>
+        </is>
+      </c>
+      <c r="CE8" t="inlineStr">
+        <is>
+          <t>$1.99</t>
+        </is>
+      </c>
+      <c r="CF8" t="inlineStr">
+        <is>
+          <t>Hy-Vee Light Bartlett Pear Halves In Pear Juice From Concentrate</t>
+        </is>
+      </c>
+      <c r="CG8" t="inlineStr">
+        <is>
+          <t>$1.69</t>
+        </is>
+      </c>
+      <c r="CH8" t="inlineStr">
+        <is>
+          <t>Hy-Vee Light Bartlett Pear Halves In Pear Juice From Concentrate</t>
+        </is>
+      </c>
+      <c r="CI8" t="inlineStr">
+        <is>
+          <t>$1.69</t>
+        </is>
+      </c>
+      <c r="CJ8" t="inlineStr">
+        <is>
+          <t>Hy-Vee Light Bartlett Pear Halves In Pear Juice From Concentrate</t>
+        </is>
+      </c>
+      <c r="CK8" t="inlineStr">
+        <is>
+          <t>$1.69</t>
+        </is>
+      </c>
+      <c r="CL8" t="inlineStr">
+        <is>
+          <t>Hy-Vee Light Bartlett Pear Halves In Pear Juice From Concentrate</t>
+        </is>
+      </c>
+      <c r="CM8" t="inlineStr">
+        <is>
+          <t>$1.69</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -3010,6 +4370,176 @@
           <t>$3.99</t>
         </is>
       </c>
+      <c r="BF9" t="inlineStr">
+        <is>
+          <t>Dole Fresh Romaine Hearts</t>
+        </is>
+      </c>
+      <c r="BG9" t="inlineStr">
+        <is>
+          <t>$3.99</t>
+        </is>
+      </c>
+      <c r="BH9" t="inlineStr">
+        <is>
+          <t>Dole Fresh Romaine Hearts</t>
+        </is>
+      </c>
+      <c r="BI9" t="inlineStr">
+        <is>
+          <t>$3.99</t>
+        </is>
+      </c>
+      <c r="BJ9" t="inlineStr">
+        <is>
+          <t>Dole Fresh Romaine Hearts</t>
+        </is>
+      </c>
+      <c r="BK9" t="inlineStr">
+        <is>
+          <t>$3.99</t>
+        </is>
+      </c>
+      <c r="BL9" t="inlineStr">
+        <is>
+          <t>Dole Fresh Romaine Hearts</t>
+        </is>
+      </c>
+      <c r="BM9" t="inlineStr">
+        <is>
+          <t>$3.99</t>
+        </is>
+      </c>
+      <c r="BN9" t="inlineStr">
+        <is>
+          <t>Dole Fresh Romaine Hearts</t>
+        </is>
+      </c>
+      <c r="BO9" t="inlineStr">
+        <is>
+          <t>$3.99</t>
+        </is>
+      </c>
+      <c r="BP9" t="inlineStr">
+        <is>
+          <t>Dole Fresh Romaine Hearts</t>
+        </is>
+      </c>
+      <c r="BQ9" t="inlineStr">
+        <is>
+          <t>$3.99</t>
+        </is>
+      </c>
+      <c r="BR9" t="inlineStr">
+        <is>
+          <t>Dole Fresh Romaine Hearts</t>
+        </is>
+      </c>
+      <c r="BS9" t="inlineStr">
+        <is>
+          <t>$3.99</t>
+        </is>
+      </c>
+      <c r="BT9" t="inlineStr">
+        <is>
+          <t>Dole Fresh Romaine Hearts</t>
+        </is>
+      </c>
+      <c r="BU9" t="inlineStr">
+        <is>
+          <t>$3.99</t>
+        </is>
+      </c>
+      <c r="BV9" t="inlineStr">
+        <is>
+          <t>Dole Fresh Romaine Hearts</t>
+        </is>
+      </c>
+      <c r="BW9" t="inlineStr">
+        <is>
+          <t>$3.99</t>
+        </is>
+      </c>
+      <c r="BX9" t="inlineStr">
+        <is>
+          <t>Dole Fresh Romaine Hearts</t>
+        </is>
+      </c>
+      <c r="BY9" t="inlineStr">
+        <is>
+          <t>$3.99</t>
+        </is>
+      </c>
+      <c r="BZ9" t="inlineStr">
+        <is>
+          <t>Dole Fresh Romaine Hearts</t>
+        </is>
+      </c>
+      <c r="CA9" t="inlineStr">
+        <is>
+          <t>$3.99</t>
+        </is>
+      </c>
+      <c r="CB9" t="inlineStr">
+        <is>
+          <t>Dole Fresh Romaine Hearts</t>
+        </is>
+      </c>
+      <c r="CC9" t="inlineStr">
+        <is>
+          <t>$3.99</t>
+        </is>
+      </c>
+      <c r="CD9" t="inlineStr">
+        <is>
+          <t>Dole Fresh Romaine Hearts</t>
+        </is>
+      </c>
+      <c r="CE9" t="inlineStr">
+        <is>
+          <t>$3.99</t>
+        </is>
+      </c>
+      <c r="CF9" t="inlineStr">
+        <is>
+          <t>Dole Fresh Romaine Hearts</t>
+        </is>
+      </c>
+      <c r="CG9" t="inlineStr">
+        <is>
+          <t>$3.99</t>
+        </is>
+      </c>
+      <c r="CH9" t="inlineStr">
+        <is>
+          <t>Dole Fresh Romaine Hearts</t>
+        </is>
+      </c>
+      <c r="CI9" t="inlineStr">
+        <is>
+          <t>$3.99</t>
+        </is>
+      </c>
+      <c r="CJ9" t="inlineStr">
+        <is>
+          <t>Dole Fresh Romaine Hearts</t>
+        </is>
+      </c>
+      <c r="CK9" t="inlineStr">
+        <is>
+          <t>$3.99</t>
+        </is>
+      </c>
+      <c r="CL9" t="inlineStr">
+        <is>
+          <t>Dole Fresh Romaine Hearts</t>
+        </is>
+      </c>
+      <c r="CM9" t="inlineStr">
+        <is>
+          <t>$3.99</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -3297,6 +4827,176 @@
           <t>$5.79</t>
         </is>
       </c>
+      <c r="BF10" t="inlineStr">
+        <is>
+          <t>Hy-Vee Oven Roasted Cured Turkey Breast &amp; White Turkey Shaved Slices</t>
+        </is>
+      </c>
+      <c r="BG10" t="inlineStr">
+        <is>
+          <t>$5.79</t>
+        </is>
+      </c>
+      <c r="BH10" t="inlineStr">
+        <is>
+          <t>Hy-Vee Oven Roasted Cured Turkey Breast &amp; White Turkey Shaved Slices</t>
+        </is>
+      </c>
+      <c r="BI10" t="inlineStr">
+        <is>
+          <t>$5.79</t>
+        </is>
+      </c>
+      <c r="BJ10" t="inlineStr">
+        <is>
+          <t>Hy-Vee Oven Roasted Cured Turkey Breast &amp; White Turkey Shaved Slices</t>
+        </is>
+      </c>
+      <c r="BK10" t="inlineStr">
+        <is>
+          <t>$5.79</t>
+        </is>
+      </c>
+      <c r="BL10" t="inlineStr">
+        <is>
+          <t>Hy-Vee Oven Roasted Cured Turkey Breast &amp; White Turkey Shaved Slices</t>
+        </is>
+      </c>
+      <c r="BM10" t="inlineStr">
+        <is>
+          <t>$5.79</t>
+        </is>
+      </c>
+      <c r="BN10" t="inlineStr">
+        <is>
+          <t>Hy-Vee Oven Roasted Cured Turkey Breast &amp; White Turkey Shaved Slices</t>
+        </is>
+      </c>
+      <c r="BO10" t="inlineStr">
+        <is>
+          <t>$5.79</t>
+        </is>
+      </c>
+      <c r="BP10" t="inlineStr">
+        <is>
+          <t>Hy-Vee Oven Roasted Cured Turkey Breast &amp; White Turkey Shaved Slices</t>
+        </is>
+      </c>
+      <c r="BQ10" t="inlineStr">
+        <is>
+          <t>$5.79</t>
+        </is>
+      </c>
+      <c r="BR10" t="inlineStr">
+        <is>
+          <t>Hy-Vee Oven Roasted Cured Turkey Breast &amp; White Turkey Shaved Slices</t>
+        </is>
+      </c>
+      <c r="BS10" t="inlineStr">
+        <is>
+          <t>$5.79</t>
+        </is>
+      </c>
+      <c r="BT10" t="inlineStr">
+        <is>
+          <t>Hy-Vee Oven Roasted Cured Turkey Breast &amp; White Turkey Shaved Slices</t>
+        </is>
+      </c>
+      <c r="BU10" t="inlineStr">
+        <is>
+          <t>$5.79</t>
+        </is>
+      </c>
+      <c r="BV10" t="inlineStr">
+        <is>
+          <t>Hy-Vee Oven Roasted Cured Turkey Breast &amp; White Turkey Shaved Slices</t>
+        </is>
+      </c>
+      <c r="BW10" t="inlineStr">
+        <is>
+          <t>$5.79</t>
+        </is>
+      </c>
+      <c r="BX10" t="inlineStr">
+        <is>
+          <t>Hy-Vee Oven Roasted Cured Turkey Breast &amp; White Turkey Shaved Slices</t>
+        </is>
+      </c>
+      <c r="BY10" t="inlineStr">
+        <is>
+          <t>$5.79</t>
+        </is>
+      </c>
+      <c r="BZ10" t="inlineStr">
+        <is>
+          <t>Hy-Vee Oven Roasted Cured Turkey Breast &amp; White Turkey Shaved Slices</t>
+        </is>
+      </c>
+      <c r="CA10" t="inlineStr">
+        <is>
+          <t>$5.79</t>
+        </is>
+      </c>
+      <c r="CB10" t="inlineStr">
+        <is>
+          <t>Hy-Vee Oven Roasted Cured Turkey Breast &amp; White Turkey Shaved Slices</t>
+        </is>
+      </c>
+      <c r="CC10" t="inlineStr">
+        <is>
+          <t>$5.79</t>
+        </is>
+      </c>
+      <c r="CD10" t="inlineStr">
+        <is>
+          <t>Hy-Vee Oven Roasted Cured Turkey Breast &amp; White Turkey Shaved Slices</t>
+        </is>
+      </c>
+      <c r="CE10" t="inlineStr">
+        <is>
+          <t>$5.79</t>
+        </is>
+      </c>
+      <c r="CF10" t="inlineStr">
+        <is>
+          <t>Hy-Vee Oven Roasted Cured Turkey Breast &amp; White Turkey Shaved Slices</t>
+        </is>
+      </c>
+      <c r="CG10" t="inlineStr">
+        <is>
+          <t>$5.79</t>
+        </is>
+      </c>
+      <c r="CH10" t="inlineStr">
+        <is>
+          <t>Hy-Vee Oven Roasted Cured Turkey Breast &amp; White Turkey Shaved Slices</t>
+        </is>
+      </c>
+      <c r="CI10" t="inlineStr">
+        <is>
+          <t>$5.79</t>
+        </is>
+      </c>
+      <c r="CJ10" t="inlineStr">
+        <is>
+          <t>Hy-Vee Oven Roasted Cured Turkey Breast &amp; White Turkey Shaved Slices</t>
+        </is>
+      </c>
+      <c r="CK10" t="inlineStr">
+        <is>
+          <t>$5.79</t>
+        </is>
+      </c>
+      <c r="CL10" t="inlineStr">
+        <is>
+          <t>Hy-Vee Oven Roasted Cured Turkey Breast &amp; White Turkey Shaved Slices</t>
+        </is>
+      </c>
+      <c r="CM10" t="inlineStr">
+        <is>
+          <t>$5.79</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -3584,6 +5284,176 @@
           <t>$2.99</t>
         </is>
       </c>
+      <c r="BF11" t="inlineStr">
+        <is>
+          <t>That's Smart! Small Curd Cottage Cheese 4% Milkfat</t>
+        </is>
+      </c>
+      <c r="BG11" t="inlineStr">
+        <is>
+          <t>$2.99</t>
+        </is>
+      </c>
+      <c r="BH11" t="inlineStr">
+        <is>
+          <t>That's Smart! Small Curd Cottage Cheese 4% Milkfat</t>
+        </is>
+      </c>
+      <c r="BI11" t="inlineStr">
+        <is>
+          <t>$2.99</t>
+        </is>
+      </c>
+      <c r="BJ11" t="inlineStr">
+        <is>
+          <t>That's Smart! Small Curd Cottage Cheese 4% Milkfat</t>
+        </is>
+      </c>
+      <c r="BK11" t="inlineStr">
+        <is>
+          <t>$2.99</t>
+        </is>
+      </c>
+      <c r="BL11" t="inlineStr">
+        <is>
+          <t>That's Smart! Small Curd Cottage Cheese 4% Milkfat</t>
+        </is>
+      </c>
+      <c r="BM11" t="inlineStr">
+        <is>
+          <t>$2.99</t>
+        </is>
+      </c>
+      <c r="BN11" t="inlineStr">
+        <is>
+          <t>That's Smart! Small Curd Cottage Cheese 4% Milkfat</t>
+        </is>
+      </c>
+      <c r="BO11" t="inlineStr">
+        <is>
+          <t>$2.99</t>
+        </is>
+      </c>
+      <c r="BP11" t="inlineStr">
+        <is>
+          <t>That's Smart! Small Curd Cottage Cheese 4% Milkfat</t>
+        </is>
+      </c>
+      <c r="BQ11" t="inlineStr">
+        <is>
+          <t>$2.99</t>
+        </is>
+      </c>
+      <c r="BR11" t="inlineStr">
+        <is>
+          <t>That's Smart! Small Curd Cottage Cheese 4% Milkfat</t>
+        </is>
+      </c>
+      <c r="BS11" t="inlineStr">
+        <is>
+          <t>$2.99</t>
+        </is>
+      </c>
+      <c r="BT11" t="inlineStr">
+        <is>
+          <t>That's Smart! Small Curd Cottage Cheese 4% Milkfat</t>
+        </is>
+      </c>
+      <c r="BU11" t="inlineStr">
+        <is>
+          <t>$2.99</t>
+        </is>
+      </c>
+      <c r="BV11" t="inlineStr">
+        <is>
+          <t>That's Smart! Small Curd Cottage Cheese 4% Milkfat</t>
+        </is>
+      </c>
+      <c r="BW11" t="inlineStr">
+        <is>
+          <t>$2.99</t>
+        </is>
+      </c>
+      <c r="BX11" t="inlineStr">
+        <is>
+          <t>That's Smart! Small Curd Cottage Cheese 4% Milkfat</t>
+        </is>
+      </c>
+      <c r="BY11" t="inlineStr">
+        <is>
+          <t>$2.99</t>
+        </is>
+      </c>
+      <c r="BZ11" t="inlineStr">
+        <is>
+          <t>That's Smart! Small Curd Cottage Cheese 4% Milkfat</t>
+        </is>
+      </c>
+      <c r="CA11" t="inlineStr">
+        <is>
+          <t>$2.99</t>
+        </is>
+      </c>
+      <c r="CB11" t="inlineStr">
+        <is>
+          <t>That's Smart! Small Curd Cottage Cheese 4% Milkfat</t>
+        </is>
+      </c>
+      <c r="CC11" t="inlineStr">
+        <is>
+          <t>$3.29</t>
+        </is>
+      </c>
+      <c r="CD11" t="inlineStr">
+        <is>
+          <t>That's Smart! Small Curd Cottage Cheese 4% Milkfat</t>
+        </is>
+      </c>
+      <c r="CE11" t="inlineStr">
+        <is>
+          <t>$3.29</t>
+        </is>
+      </c>
+      <c r="CF11" t="inlineStr">
+        <is>
+          <t>That's Smart! Small Curd Cottage Cheese 4% Milkfat</t>
+        </is>
+      </c>
+      <c r="CG11" t="inlineStr">
+        <is>
+          <t>$3.29</t>
+        </is>
+      </c>
+      <c r="CH11" t="inlineStr">
+        <is>
+          <t>That's Smart! Small Curd Cottage Cheese 4% Milkfat</t>
+        </is>
+      </c>
+      <c r="CI11" t="inlineStr">
+        <is>
+          <t>$3.29</t>
+        </is>
+      </c>
+      <c r="CJ11" t="inlineStr">
+        <is>
+          <t>That's Smart! Small Curd Cottage Cheese 4% Milkfat</t>
+        </is>
+      </c>
+      <c r="CK11" t="inlineStr">
+        <is>
+          <t>$3.29</t>
+        </is>
+      </c>
+      <c r="CL11" t="inlineStr">
+        <is>
+          <t>That's Smart! Small Curd Cottage Cheese 4% Milkfat</t>
+        </is>
+      </c>
+      <c r="CM11" t="inlineStr">
+        <is>
+          <t>$3.29</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -3871,6 +5741,176 @@
           <t>$4.97</t>
         </is>
       </c>
+      <c r="BF12" t="inlineStr">
+        <is>
+          <t>Fairlife Fat Free Ultra-Filtered Milk</t>
+        </is>
+      </c>
+      <c r="BG12" t="inlineStr">
+        <is>
+          <t>$4.97</t>
+        </is>
+      </c>
+      <c r="BH12" t="inlineStr">
+        <is>
+          <t>Fairlife Fat Free Ultra-Filtered Milk</t>
+        </is>
+      </c>
+      <c r="BI12" t="inlineStr">
+        <is>
+          <t>$4.97</t>
+        </is>
+      </c>
+      <c r="BJ12" t="inlineStr">
+        <is>
+          <t>Fairlife Fat Free Ultra-Filtered Milk</t>
+        </is>
+      </c>
+      <c r="BK12" t="inlineStr">
+        <is>
+          <t>$4.97</t>
+        </is>
+      </c>
+      <c r="BL12" t="inlineStr">
+        <is>
+          <t>Fairlife Fat Free Ultra-Filtered Milk</t>
+        </is>
+      </c>
+      <c r="BM12" t="inlineStr">
+        <is>
+          <t>$4.97</t>
+        </is>
+      </c>
+      <c r="BN12" t="inlineStr">
+        <is>
+          <t>Fairlife Fat Free Ultra-Filtered Milk</t>
+        </is>
+      </c>
+      <c r="BO12" t="inlineStr">
+        <is>
+          <t>$4.97</t>
+        </is>
+      </c>
+      <c r="BP12" t="inlineStr">
+        <is>
+          <t>Fairlife Fat Free Ultra-Filtered Milk</t>
+        </is>
+      </c>
+      <c r="BQ12" t="inlineStr">
+        <is>
+          <t>$4.97</t>
+        </is>
+      </c>
+      <c r="BR12" t="inlineStr">
+        <is>
+          <t>Fairlife Fat Free Ultra-Filtered Milk</t>
+        </is>
+      </c>
+      <c r="BS12" t="inlineStr">
+        <is>
+          <t>$4.97</t>
+        </is>
+      </c>
+      <c r="BT12" t="inlineStr">
+        <is>
+          <t>Fairlife Fat Free Ultra-Filtered Milk</t>
+        </is>
+      </c>
+      <c r="BU12" t="inlineStr">
+        <is>
+          <t>$4.97</t>
+        </is>
+      </c>
+      <c r="BV12" t="inlineStr">
+        <is>
+          <t>Fairlife Fat Free Ultra-Filtered Milk</t>
+        </is>
+      </c>
+      <c r="BW12" t="inlineStr">
+        <is>
+          <t>$4.97</t>
+        </is>
+      </c>
+      <c r="BX12" t="inlineStr">
+        <is>
+          <t>Fairlife Fat Free Ultra-Filtered Milk</t>
+        </is>
+      </c>
+      <c r="BY12" t="inlineStr">
+        <is>
+          <t>$4.97</t>
+        </is>
+      </c>
+      <c r="BZ12" t="inlineStr">
+        <is>
+          <t>Fairlife Fat Free Ultra-Filtered Milk</t>
+        </is>
+      </c>
+      <c r="CA12" t="inlineStr">
+        <is>
+          <t>$4.97</t>
+        </is>
+      </c>
+      <c r="CB12" t="inlineStr">
+        <is>
+          <t>Fairlife Fat Free Ultra-Filtered Milk</t>
+        </is>
+      </c>
+      <c r="CC12" t="inlineStr">
+        <is>
+          <t>$4.97</t>
+        </is>
+      </c>
+      <c r="CD12" t="inlineStr">
+        <is>
+          <t>Fairlife Fat Free Ultra-Filtered Milk</t>
+        </is>
+      </c>
+      <c r="CE12" t="inlineStr">
+        <is>
+          <t>$4.97</t>
+        </is>
+      </c>
+      <c r="CF12" t="inlineStr">
+        <is>
+          <t>Fairlife Fat Free Ultra-Filtered Milk</t>
+        </is>
+      </c>
+      <c r="CG12" t="inlineStr">
+        <is>
+          <t>$4.97</t>
+        </is>
+      </c>
+      <c r="CH12" t="inlineStr">
+        <is>
+          <t>Fairlife Fat Free Ultra-Filtered Milk</t>
+        </is>
+      </c>
+      <c r="CI12" t="inlineStr">
+        <is>
+          <t>$4.97</t>
+        </is>
+      </c>
+      <c r="CJ12" t="inlineStr">
+        <is>
+          <t>Fairlife Fat Free Ultra-Filtered Milk</t>
+        </is>
+      </c>
+      <c r="CK12" t="inlineStr">
+        <is>
+          <t>$4.97</t>
+        </is>
+      </c>
+      <c r="CL12" t="inlineStr">
+        <is>
+          <t>Fairlife Fat Free Ultra-Filtered Milk</t>
+        </is>
+      </c>
+      <c r="CM12" t="inlineStr">
+        <is>
+          <t>$4.97</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -4158,6 +6198,176 @@
           <t>16¢ ea.</t>
         </is>
       </c>
+      <c r="BF13" t="inlineStr">
+        <is>
+          <t>Fresh Chiquita Bananas</t>
+        </is>
+      </c>
+      <c r="BG13" t="inlineStr">
+        <is>
+          <t>16¢ ea.</t>
+        </is>
+      </c>
+      <c r="BH13" t="inlineStr">
+        <is>
+          <t>Fresh Chiquita Bananas</t>
+        </is>
+      </c>
+      <c r="BI13" t="inlineStr">
+        <is>
+          <t>16¢ ea.</t>
+        </is>
+      </c>
+      <c r="BJ13" t="inlineStr">
+        <is>
+          <t>Fresh Chiquita Bananas</t>
+        </is>
+      </c>
+      <c r="BK13" t="inlineStr">
+        <is>
+          <t>16¢ ea.</t>
+        </is>
+      </c>
+      <c r="BL13" t="inlineStr">
+        <is>
+          <t>Fresh Chiquita Bananas</t>
+        </is>
+      </c>
+      <c r="BM13" t="inlineStr">
+        <is>
+          <t>16¢ ea.</t>
+        </is>
+      </c>
+      <c r="BN13" t="inlineStr">
+        <is>
+          <t>Fresh Chiquita Bananas</t>
+        </is>
+      </c>
+      <c r="BO13" t="inlineStr">
+        <is>
+          <t>16¢ ea.</t>
+        </is>
+      </c>
+      <c r="BP13" t="inlineStr">
+        <is>
+          <t>Fresh Chiquita Bananas</t>
+        </is>
+      </c>
+      <c r="BQ13" t="inlineStr">
+        <is>
+          <t>16¢ ea.</t>
+        </is>
+      </c>
+      <c r="BR13" t="inlineStr">
+        <is>
+          <t>Fresh Chiquita Bananas</t>
+        </is>
+      </c>
+      <c r="BS13" t="inlineStr">
+        <is>
+          <t>16¢ ea.</t>
+        </is>
+      </c>
+      <c r="BT13" t="inlineStr">
+        <is>
+          <t>Fresh Chiquita Bananas</t>
+        </is>
+      </c>
+      <c r="BU13" t="inlineStr">
+        <is>
+          <t>16¢ ea.</t>
+        </is>
+      </c>
+      <c r="BV13" t="inlineStr">
+        <is>
+          <t>Fresh Chiquita Bananas</t>
+        </is>
+      </c>
+      <c r="BW13" t="inlineStr">
+        <is>
+          <t>16¢ ea.</t>
+        </is>
+      </c>
+      <c r="BX13" t="inlineStr">
+        <is>
+          <t>Fresh Chiquita Bananas</t>
+        </is>
+      </c>
+      <c r="BY13" t="inlineStr">
+        <is>
+          <t>16¢ ea.</t>
+        </is>
+      </c>
+      <c r="BZ13" t="inlineStr">
+        <is>
+          <t>Fresh Chiquita Bananas</t>
+        </is>
+      </c>
+      <c r="CA13" t="inlineStr">
+        <is>
+          <t>16¢ ea.</t>
+        </is>
+      </c>
+      <c r="CB13" t="inlineStr">
+        <is>
+          <t>Fresh Chiquita Bananas</t>
+        </is>
+      </c>
+      <c r="CC13" t="inlineStr">
+        <is>
+          <t>16¢ ea.</t>
+        </is>
+      </c>
+      <c r="CD13" t="inlineStr">
+        <is>
+          <t>Fresh Chiquita Bananas</t>
+        </is>
+      </c>
+      <c r="CE13" t="inlineStr">
+        <is>
+          <t>16¢ ea.</t>
+        </is>
+      </c>
+      <c r="CF13" t="inlineStr">
+        <is>
+          <t>Fresh Chiquita Bananas</t>
+        </is>
+      </c>
+      <c r="CG13" t="inlineStr">
+        <is>
+          <t>16¢ ea.</t>
+        </is>
+      </c>
+      <c r="CH13" t="inlineStr">
+        <is>
+          <t>Fresh Chiquita Bananas</t>
+        </is>
+      </c>
+      <c r="CI13" t="inlineStr">
+        <is>
+          <t>16¢ ea.</t>
+        </is>
+      </c>
+      <c r="CJ13" t="inlineStr">
+        <is>
+          <t>Fresh Chiquita Bananas</t>
+        </is>
+      </c>
+      <c r="CK13" t="inlineStr">
+        <is>
+          <t>16¢ ea.</t>
+        </is>
+      </c>
+      <c r="CL13" t="inlineStr">
+        <is>
+          <t>Fresh Chiquita Bananas</t>
+        </is>
+      </c>
+      <c r="CM13" t="inlineStr">
+        <is>
+          <t>16¢ ea.</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -4445,6 +6655,176 @@
           <t>$5.89</t>
         </is>
       </c>
+      <c r="BF14" t="inlineStr">
+        <is>
+          <t>Wonderful Halos Mandarin Oranges</t>
+        </is>
+      </c>
+      <c r="BG14" t="inlineStr">
+        <is>
+          <t>$5.89</t>
+        </is>
+      </c>
+      <c r="BH14" t="inlineStr">
+        <is>
+          <t>Wonderful Halos Mandarin Oranges</t>
+        </is>
+      </c>
+      <c r="BI14" t="inlineStr">
+        <is>
+          <t>$5.89</t>
+        </is>
+      </c>
+      <c r="BJ14" t="inlineStr">
+        <is>
+          <t>Wonderful Halos Mandarin Oranges</t>
+        </is>
+      </c>
+      <c r="BK14" t="inlineStr">
+        <is>
+          <t>$5.89</t>
+        </is>
+      </c>
+      <c r="BL14" t="inlineStr">
+        <is>
+          <t>Wonderful Halos Mandarin Oranges</t>
+        </is>
+      </c>
+      <c r="BM14" t="inlineStr">
+        <is>
+          <t>$5.89</t>
+        </is>
+      </c>
+      <c r="BN14" t="inlineStr">
+        <is>
+          <t>Wonderful Halos Mandarin Oranges</t>
+        </is>
+      </c>
+      <c r="BO14" t="inlineStr">
+        <is>
+          <t>$5.89</t>
+        </is>
+      </c>
+      <c r="BP14" t="inlineStr">
+        <is>
+          <t>Wonderful Halos Mandarin Oranges</t>
+        </is>
+      </c>
+      <c r="BQ14" t="inlineStr">
+        <is>
+          <t>$5.89</t>
+        </is>
+      </c>
+      <c r="BR14" t="inlineStr">
+        <is>
+          <t>Wonderful Halos Mandarin Oranges</t>
+        </is>
+      </c>
+      <c r="BS14" t="inlineStr">
+        <is>
+          <t>$5.89</t>
+        </is>
+      </c>
+      <c r="BT14" t="inlineStr">
+        <is>
+          <t>Wonderful Halos Mandarin Oranges</t>
+        </is>
+      </c>
+      <c r="BU14" t="inlineStr">
+        <is>
+          <t>$5.89</t>
+        </is>
+      </c>
+      <c r="BV14" t="inlineStr">
+        <is>
+          <t>Wonderful Halos Mandarin Oranges</t>
+        </is>
+      </c>
+      <c r="BW14" t="inlineStr">
+        <is>
+          <t>$5.89</t>
+        </is>
+      </c>
+      <c r="BX14" t="inlineStr">
+        <is>
+          <t>Wonderful Halos Mandarin Oranges</t>
+        </is>
+      </c>
+      <c r="BY14" t="inlineStr">
+        <is>
+          <t>$5.89</t>
+        </is>
+      </c>
+      <c r="BZ14" t="inlineStr">
+        <is>
+          <t>Wonderful Halos Mandarin Oranges</t>
+        </is>
+      </c>
+      <c r="CA14" t="inlineStr">
+        <is>
+          <t>$3.99</t>
+        </is>
+      </c>
+      <c r="CB14" t="inlineStr">
+        <is>
+          <t>Wonderful Halos Mandarin Oranges</t>
+        </is>
+      </c>
+      <c r="CC14" t="inlineStr">
+        <is>
+          <t>$5.89</t>
+        </is>
+      </c>
+      <c r="CD14" t="inlineStr">
+        <is>
+          <t>Wonderful Halos Mandarin Oranges</t>
+        </is>
+      </c>
+      <c r="CE14" t="inlineStr">
+        <is>
+          <t>$5.89</t>
+        </is>
+      </c>
+      <c r="CF14" t="inlineStr">
+        <is>
+          <t>Wonderful Halos Mandarin Oranges</t>
+        </is>
+      </c>
+      <c r="CG14" t="inlineStr">
+        <is>
+          <t>$5.89</t>
+        </is>
+      </c>
+      <c r="CH14" t="inlineStr">
+        <is>
+          <t>Wonderful Halos Mandarin Oranges</t>
+        </is>
+      </c>
+      <c r="CI14" t="inlineStr">
+        <is>
+          <t>$5.89</t>
+        </is>
+      </c>
+      <c r="CJ14" t="inlineStr">
+        <is>
+          <t>Wonderful Halos Mandarin Oranges</t>
+        </is>
+      </c>
+      <c r="CK14" t="inlineStr">
+        <is>
+          <t>$5.89</t>
+        </is>
+      </c>
+      <c r="CL14" t="inlineStr">
+        <is>
+          <t>Wonderful Halos Mandarin Oranges</t>
+        </is>
+      </c>
+      <c r="CM14" t="inlineStr">
+        <is>
+          <t>$5.89</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -4732,6 +7112,176 @@
           <t>$6.99/lb</t>
         </is>
       </c>
+      <c r="BF15" t="inlineStr">
+        <is>
+          <t>Certified Ground Round 90% Lean 10% Fat</t>
+        </is>
+      </c>
+      <c r="BG15" t="inlineStr">
+        <is>
+          <t>$6.99/lb</t>
+        </is>
+      </c>
+      <c r="BH15" t="inlineStr">
+        <is>
+          <t>Certified Ground Round 90% Lean 10% Fat</t>
+        </is>
+      </c>
+      <c r="BI15" t="inlineStr">
+        <is>
+          <t>$6.99/lb</t>
+        </is>
+      </c>
+      <c r="BJ15" t="inlineStr">
+        <is>
+          <t>Certified Ground Round 90% Lean 10% Fat</t>
+        </is>
+      </c>
+      <c r="BK15" t="inlineStr">
+        <is>
+          <t>$6.99/lb</t>
+        </is>
+      </c>
+      <c r="BL15" t="inlineStr">
+        <is>
+          <t>Certified Ground Round 90% Lean 10% Fat</t>
+        </is>
+      </c>
+      <c r="BM15" t="inlineStr">
+        <is>
+          <t>$6.99/lb</t>
+        </is>
+      </c>
+      <c r="BN15" t="inlineStr">
+        <is>
+          <t>Certified Ground Round 90% Lean 10% Fat</t>
+        </is>
+      </c>
+      <c r="BO15" t="inlineStr">
+        <is>
+          <t>$6.99/lb</t>
+        </is>
+      </c>
+      <c r="BP15" t="inlineStr">
+        <is>
+          <t>Certified Ground Round 90% Lean 10% Fat</t>
+        </is>
+      </c>
+      <c r="BQ15" t="inlineStr">
+        <is>
+          <t>$6.99/lb</t>
+        </is>
+      </c>
+      <c r="BR15" t="inlineStr">
+        <is>
+          <t>Certified Ground Round 90% Lean 10% Fat</t>
+        </is>
+      </c>
+      <c r="BS15" t="inlineStr">
+        <is>
+          <t>$6.99/lb</t>
+        </is>
+      </c>
+      <c r="BT15" t="inlineStr">
+        <is>
+          <t>Certified Ground Round 90% Lean 10% Fat</t>
+        </is>
+      </c>
+      <c r="BU15" t="inlineStr">
+        <is>
+          <t>$6.99/lb</t>
+        </is>
+      </c>
+      <c r="BV15" t="inlineStr">
+        <is>
+          <t>Certified Ground Round 90% Lean 10% Fat</t>
+        </is>
+      </c>
+      <c r="BW15" t="inlineStr">
+        <is>
+          <t>$6.99/lb</t>
+        </is>
+      </c>
+      <c r="BX15" t="inlineStr">
+        <is>
+          <t>Certified Ground Round 90% Lean 10% Fat</t>
+        </is>
+      </c>
+      <c r="BY15" t="inlineStr">
+        <is>
+          <t>$6.99/lb</t>
+        </is>
+      </c>
+      <c r="BZ15" t="inlineStr">
+        <is>
+          <t>Certified Ground Round 90% Lean 10% Fat</t>
+        </is>
+      </c>
+      <c r="CA15" t="inlineStr">
+        <is>
+          <t>$6.99/lb</t>
+        </is>
+      </c>
+      <c r="CB15" t="inlineStr">
+        <is>
+          <t>Certified Ground Round 90% Lean 10% Fat</t>
+        </is>
+      </c>
+      <c r="CC15" t="inlineStr">
+        <is>
+          <t>$6.99/lb</t>
+        </is>
+      </c>
+      <c r="CD15" t="inlineStr">
+        <is>
+          <t>Certified Ground Round 90% Lean 10% Fat</t>
+        </is>
+      </c>
+      <c r="CE15" t="inlineStr">
+        <is>
+          <t>$6.99/lb</t>
+        </is>
+      </c>
+      <c r="CF15" t="inlineStr">
+        <is>
+          <t>Certified Ground Round 90% Lean 10% Fat</t>
+        </is>
+      </c>
+      <c r="CG15" t="inlineStr">
+        <is>
+          <t>$6.99/lb</t>
+        </is>
+      </c>
+      <c r="CH15" t="inlineStr">
+        <is>
+          <t>Certified Ground Round 90% Lean 10% Fat</t>
+        </is>
+      </c>
+      <c r="CI15" t="inlineStr">
+        <is>
+          <t>$6.99/lb</t>
+        </is>
+      </c>
+      <c r="CJ15" t="inlineStr">
+        <is>
+          <t>Certified Ground Round 90% Lean 10% Fat</t>
+        </is>
+      </c>
+      <c r="CK15" t="inlineStr">
+        <is>
+          <t>$6.99/lb</t>
+        </is>
+      </c>
+      <c r="CL15" t="inlineStr">
+        <is>
+          <t>Certified Ground Round 90% Lean 10% Fat</t>
+        </is>
+      </c>
+      <c r="CM15" t="inlineStr">
+        <is>
+          <t>$6.99/lb</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -5019,6 +7569,176 @@
           <t>$3.83 ea.</t>
         </is>
       </c>
+      <c r="BF16" t="inlineStr">
+        <is>
+          <t>Boneless Skinless Chicken Breast</t>
+        </is>
+      </c>
+      <c r="BG16" t="inlineStr">
+        <is>
+          <t>$3.83 ea.</t>
+        </is>
+      </c>
+      <c r="BH16" t="inlineStr">
+        <is>
+          <t>Boneless Skinless Chicken Breast</t>
+        </is>
+      </c>
+      <c r="BI16" t="inlineStr">
+        <is>
+          <t>$3.83 ea.</t>
+        </is>
+      </c>
+      <c r="BJ16" t="inlineStr">
+        <is>
+          <t>Boneless Skinless Chicken Breast</t>
+        </is>
+      </c>
+      <c r="BK16" t="inlineStr">
+        <is>
+          <t>$3.83 ea.</t>
+        </is>
+      </c>
+      <c r="BL16" t="inlineStr">
+        <is>
+          <t>Boneless Skinless Chicken Breast</t>
+        </is>
+      </c>
+      <c r="BM16" t="inlineStr">
+        <is>
+          <t>$3.83 ea.</t>
+        </is>
+      </c>
+      <c r="BN16" t="inlineStr">
+        <is>
+          <t>Boneless Skinless Chicken Breast</t>
+        </is>
+      </c>
+      <c r="BO16" t="inlineStr">
+        <is>
+          <t>$3.83 ea.</t>
+        </is>
+      </c>
+      <c r="BP16" t="inlineStr">
+        <is>
+          <t>Boneless Skinless Chicken Breast</t>
+        </is>
+      </c>
+      <c r="BQ16" t="inlineStr">
+        <is>
+          <t>$3.83 ea.</t>
+        </is>
+      </c>
+      <c r="BR16" t="inlineStr">
+        <is>
+          <t>Boneless Skinless Chicken Breast</t>
+        </is>
+      </c>
+      <c r="BS16" t="inlineStr">
+        <is>
+          <t>$3.83 ea.</t>
+        </is>
+      </c>
+      <c r="BT16" t="inlineStr">
+        <is>
+          <t>Boneless Skinless Chicken Breast</t>
+        </is>
+      </c>
+      <c r="BU16" t="inlineStr">
+        <is>
+          <t>$3.83 ea.</t>
+        </is>
+      </c>
+      <c r="BV16" t="inlineStr">
+        <is>
+          <t>Boneless Skinless Chicken Breast</t>
+        </is>
+      </c>
+      <c r="BW16" t="inlineStr">
+        <is>
+          <t>$3.83 ea.</t>
+        </is>
+      </c>
+      <c r="BX16" t="inlineStr">
+        <is>
+          <t>Boneless Skinless Chicken Breast</t>
+        </is>
+      </c>
+      <c r="BY16" t="inlineStr">
+        <is>
+          <t>$3.83 ea.</t>
+        </is>
+      </c>
+      <c r="BZ16" t="inlineStr">
+        <is>
+          <t>Boneless Skinless Chicken Breast</t>
+        </is>
+      </c>
+      <c r="CA16" t="inlineStr">
+        <is>
+          <t>$3.83 ea.</t>
+        </is>
+      </c>
+      <c r="CB16" t="inlineStr">
+        <is>
+          <t>Boneless Skinless Chicken Breast</t>
+        </is>
+      </c>
+      <c r="CC16" t="inlineStr">
+        <is>
+          <t>$3.83 ea.</t>
+        </is>
+      </c>
+      <c r="CD16" t="inlineStr">
+        <is>
+          <t>Boneless Skinless Chicken Breast</t>
+        </is>
+      </c>
+      <c r="CE16" t="inlineStr">
+        <is>
+          <t>$3.83 ea.</t>
+        </is>
+      </c>
+      <c r="CF16" t="inlineStr">
+        <is>
+          <t>Boneless Skinless Chicken Breast</t>
+        </is>
+      </c>
+      <c r="CG16" t="inlineStr">
+        <is>
+          <t>$3.83 ea.</t>
+        </is>
+      </c>
+      <c r="CH16" t="inlineStr">
+        <is>
+          <t>Boneless Skinless Chicken Breast</t>
+        </is>
+      </c>
+      <c r="CI16" t="inlineStr">
+        <is>
+          <t>$3.83 ea.</t>
+        </is>
+      </c>
+      <c r="CJ16" t="inlineStr">
+        <is>
+          <t>Boneless Skinless Chicken Breast</t>
+        </is>
+      </c>
+      <c r="CK16" t="inlineStr">
+        <is>
+          <t>$3.83 ea.</t>
+        </is>
+      </c>
+      <c r="CL16" t="inlineStr">
+        <is>
+          <t>Boneless Skinless Chicken Breast</t>
+        </is>
+      </c>
+      <c r="CM16" t="inlineStr">
+        <is>
+          <t>$3.83 ea.</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -5306,6 +8026,176 @@
           <t>$40,275</t>
         </is>
       </c>
+      <c r="BF17" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="BG17" t="inlineStr">
+        <is>
+          <t>$40,275</t>
+        </is>
+      </c>
+      <c r="BH17" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="BI17" t="inlineStr">
+        <is>
+          <t>$40,275</t>
+        </is>
+      </c>
+      <c r="BJ17" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="BK17" t="inlineStr">
+        <is>
+          <t>$40,275</t>
+        </is>
+      </c>
+      <c r="BL17" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="BM17" t="inlineStr">
+        <is>
+          <t>$40,275</t>
+        </is>
+      </c>
+      <c r="BN17" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="BO17" t="inlineStr">
+        <is>
+          <t>$40,275</t>
+        </is>
+      </c>
+      <c r="BP17" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="BQ17" t="inlineStr">
+        <is>
+          <t>$40,275</t>
+        </is>
+      </c>
+      <c r="BR17" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="BS17" t="inlineStr">
+        <is>
+          <t>$40,275</t>
+        </is>
+      </c>
+      <c r="BT17" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="BU17" t="inlineStr">
+        <is>
+          <t>$40,275</t>
+        </is>
+      </c>
+      <c r="BV17" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="BW17" t="inlineStr">
+        <is>
+          <t>$40,275</t>
+        </is>
+      </c>
+      <c r="BX17" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="BY17" t="inlineStr">
+        <is>
+          <t>$40,275</t>
+        </is>
+      </c>
+      <c r="BZ17" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="CA17" t="inlineStr">
+        <is>
+          <t>$40,275</t>
+        </is>
+      </c>
+      <c r="CB17" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="CC17" t="inlineStr">
+        <is>
+          <t>$40,275</t>
+        </is>
+      </c>
+      <c r="CD17" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="CE17" t="inlineStr">
+        <is>
+          <t>$40,275</t>
+        </is>
+      </c>
+      <c r="CF17" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="CG17" t="inlineStr">
+        <is>
+          <t>$40,275</t>
+        </is>
+      </c>
+      <c r="CH17" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="CI17" t="inlineStr">
+        <is>
+          <t>$40,275</t>
+        </is>
+      </c>
+      <c r="CJ17" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="CK17" t="inlineStr">
+        <is>
+          <t>$40,275</t>
+        </is>
+      </c>
+      <c r="CL17" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="CM17" t="inlineStr">
+        <is>
+          <t>$40,275</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -5477,6 +8367,108 @@
       </c>
       <c r="BD18" t="inlineStr"/>
       <c r="BE18" t="inlineStr">
+        <is>
+          <t>$37,000*</t>
+        </is>
+      </c>
+      <c r="BF18" t="inlineStr"/>
+      <c r="BG18" t="inlineStr">
+        <is>
+          <t>$37,000*</t>
+        </is>
+      </c>
+      <c r="BH18" t="inlineStr"/>
+      <c r="BI18" t="inlineStr">
+        <is>
+          <t>$37,000*</t>
+        </is>
+      </c>
+      <c r="BJ18" t="inlineStr"/>
+      <c r="BK18" t="inlineStr">
+        <is>
+          <t>$37,000*</t>
+        </is>
+      </c>
+      <c r="BL18" t="inlineStr"/>
+      <c r="BM18" t="inlineStr">
+        <is>
+          <t>$37,000*</t>
+        </is>
+      </c>
+      <c r="BN18" t="inlineStr"/>
+      <c r="BO18" t="inlineStr">
+        <is>
+          <t>$37,000*</t>
+        </is>
+      </c>
+      <c r="BP18" t="inlineStr"/>
+      <c r="BQ18" t="inlineStr">
+        <is>
+          <t>$37,000*</t>
+        </is>
+      </c>
+      <c r="BR18" t="inlineStr"/>
+      <c r="BS18" t="inlineStr">
+        <is>
+          <t>$37,000*</t>
+        </is>
+      </c>
+      <c r="BT18" t="inlineStr"/>
+      <c r="BU18" t="inlineStr">
+        <is>
+          <t>$37,000*</t>
+        </is>
+      </c>
+      <c r="BV18" t="inlineStr"/>
+      <c r="BW18" t="inlineStr">
+        <is>
+          <t>$37,000*</t>
+        </is>
+      </c>
+      <c r="BX18" t="inlineStr"/>
+      <c r="BY18" t="inlineStr">
+        <is>
+          <t>$37,000*</t>
+        </is>
+      </c>
+      <c r="BZ18" t="inlineStr"/>
+      <c r="CA18" t="inlineStr">
+        <is>
+          <t>$37,000*</t>
+        </is>
+      </c>
+      <c r="CB18" t="inlineStr"/>
+      <c r="CC18" t="inlineStr">
+        <is>
+          <t>$37,000*</t>
+        </is>
+      </c>
+      <c r="CD18" t="inlineStr"/>
+      <c r="CE18" t="inlineStr">
+        <is>
+          <t>$37,000*</t>
+        </is>
+      </c>
+      <c r="CF18" t="inlineStr"/>
+      <c r="CG18" t="inlineStr">
+        <is>
+          <t>$37,000*</t>
+        </is>
+      </c>
+      <c r="CH18" t="inlineStr"/>
+      <c r="CI18" t="inlineStr">
+        <is>
+          <t>$37,000*</t>
+        </is>
+      </c>
+      <c r="CJ18" t="inlineStr"/>
+      <c r="CK18" t="inlineStr">
+        <is>
+          <t>$37,000*</t>
+        </is>
+      </c>
+      <c r="CL18" t="inlineStr"/>
+      <c r="CM18" t="inlineStr">
         <is>
           <t>$37,000*</t>
         </is>
@@ -5684,6 +8676,108 @@
           <t>Not found</t>
         </is>
       </c>
+      <c r="BF19" t="inlineStr"/>
+      <c r="BG19" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="BH19" t="inlineStr"/>
+      <c r="BI19" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="BJ19" t="inlineStr"/>
+      <c r="BK19" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="BL19" t="inlineStr"/>
+      <c r="BM19" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="BN19" t="inlineStr"/>
+      <c r="BO19" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="BP19" t="inlineStr"/>
+      <c r="BQ19" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="BR19" t="inlineStr"/>
+      <c r="BS19" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="BT19" t="inlineStr"/>
+      <c r="BU19" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="BV19" t="inlineStr"/>
+      <c r="BW19" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="BX19" t="inlineStr"/>
+      <c r="BY19" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="BZ19" t="inlineStr"/>
+      <c r="CA19" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="CB19" t="inlineStr"/>
+      <c r="CC19" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="CD19" t="inlineStr"/>
+      <c r="CE19" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="CF19" t="inlineStr"/>
+      <c r="CG19" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="CH19" t="inlineStr"/>
+      <c r="CI19" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="CJ19" t="inlineStr"/>
+      <c r="CK19" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="CL19" t="inlineStr"/>
+      <c r="CM19" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -5971,6 +9065,176 @@
           <t>$6.99</t>
         </is>
       </c>
+      <c r="BF20" t="inlineStr">
+        <is>
+          <t>Hy-Vee Select 100% Pure Maple Syrup</t>
+        </is>
+      </c>
+      <c r="BG20" t="inlineStr">
+        <is>
+          <t>$6.99</t>
+        </is>
+      </c>
+      <c r="BH20" t="inlineStr">
+        <is>
+          <t>Hy-Vee Select 100% Pure Maple Syrup</t>
+        </is>
+      </c>
+      <c r="BI20" t="inlineStr">
+        <is>
+          <t>$6.99</t>
+        </is>
+      </c>
+      <c r="BJ20" t="inlineStr">
+        <is>
+          <t>Hy-Vee Select 100% Pure Maple Syrup</t>
+        </is>
+      </c>
+      <c r="BK20" t="inlineStr">
+        <is>
+          <t>$6.99</t>
+        </is>
+      </c>
+      <c r="BL20" t="inlineStr">
+        <is>
+          <t>Hy-Vee Select 100% Pure Maple Syrup</t>
+        </is>
+      </c>
+      <c r="BM20" t="inlineStr">
+        <is>
+          <t>$6.99</t>
+        </is>
+      </c>
+      <c r="BN20" t="inlineStr">
+        <is>
+          <t>Hy-Vee Select 100% Pure Maple Syrup</t>
+        </is>
+      </c>
+      <c r="BO20" t="inlineStr">
+        <is>
+          <t>$6.99</t>
+        </is>
+      </c>
+      <c r="BP20" t="inlineStr">
+        <is>
+          <t>Hy-Vee Select 100% Pure Maple Syrup</t>
+        </is>
+      </c>
+      <c r="BQ20" t="inlineStr">
+        <is>
+          <t>$6.99</t>
+        </is>
+      </c>
+      <c r="BR20" t="inlineStr">
+        <is>
+          <t>Hy-Vee Select 100% Pure Maple Syrup</t>
+        </is>
+      </c>
+      <c r="BS20" t="inlineStr">
+        <is>
+          <t>$6.99</t>
+        </is>
+      </c>
+      <c r="BT20" t="inlineStr">
+        <is>
+          <t>Hy-Vee Select 100% Pure Maple Syrup</t>
+        </is>
+      </c>
+      <c r="BU20" t="inlineStr">
+        <is>
+          <t>$6.99</t>
+        </is>
+      </c>
+      <c r="BV20" t="inlineStr">
+        <is>
+          <t>Hy-Vee Select 100% Pure Maple Syrup</t>
+        </is>
+      </c>
+      <c r="BW20" t="inlineStr">
+        <is>
+          <t>$6.99</t>
+        </is>
+      </c>
+      <c r="BX20" t="inlineStr">
+        <is>
+          <t>Hy-Vee Select 100% Pure Maple Syrup</t>
+        </is>
+      </c>
+      <c r="BY20" t="inlineStr">
+        <is>
+          <t>$6.99</t>
+        </is>
+      </c>
+      <c r="BZ20" t="inlineStr">
+        <is>
+          <t>Hy-Vee Select 100% Pure Maple Syrup</t>
+        </is>
+      </c>
+      <c r="CA20" t="inlineStr">
+        <is>
+          <t>$6.99</t>
+        </is>
+      </c>
+      <c r="CB20" t="inlineStr">
+        <is>
+          <t>Hy-Vee Select 100% Pure Maple Syrup</t>
+        </is>
+      </c>
+      <c r="CC20" t="inlineStr">
+        <is>
+          <t>$6.99</t>
+        </is>
+      </c>
+      <c r="CD20" t="inlineStr">
+        <is>
+          <t>Hy-Vee Select 100% Pure Maple Syrup</t>
+        </is>
+      </c>
+      <c r="CE20" t="inlineStr">
+        <is>
+          <t>$6.99</t>
+        </is>
+      </c>
+      <c r="CF20" t="inlineStr">
+        <is>
+          <t>Hy-Vee Select 100% Pure Maple Syrup</t>
+        </is>
+      </c>
+      <c r="CG20" t="inlineStr">
+        <is>
+          <t>$6.99</t>
+        </is>
+      </c>
+      <c r="CH20" t="inlineStr">
+        <is>
+          <t>Hy-Vee Select 100% Pure Maple Syrup</t>
+        </is>
+      </c>
+      <c r="CI20" t="inlineStr">
+        <is>
+          <t>$6.99</t>
+        </is>
+      </c>
+      <c r="CJ20" t="inlineStr">
+        <is>
+          <t>Hy-Vee Select 100% Pure Maple Syrup</t>
+        </is>
+      </c>
+      <c r="CK20" t="inlineStr">
+        <is>
+          <t>$6.99</t>
+        </is>
+      </c>
+      <c r="CL20" t="inlineStr">
+        <is>
+          <t>Hy-Vee Select 100% Pure Maple Syrup</t>
+        </is>
+      </c>
+      <c r="CM20" t="inlineStr">
+        <is>
+          <t>$6.99</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -6258,6 +9522,176 @@
           <t>$5.97</t>
         </is>
       </c>
+      <c r="BF21" t="inlineStr">
+        <is>
+          <t>That's Smart! Large Shell Eggs</t>
+        </is>
+      </c>
+      <c r="BG21" t="inlineStr">
+        <is>
+          <t>$5.97</t>
+        </is>
+      </c>
+      <c r="BH21" t="inlineStr">
+        <is>
+          <t>That's Smart! Large Shell Eggs</t>
+        </is>
+      </c>
+      <c r="BI21" t="inlineStr">
+        <is>
+          <t>$5.97</t>
+        </is>
+      </c>
+      <c r="BJ21" t="inlineStr">
+        <is>
+          <t>That's Smart! Large Shell Eggs</t>
+        </is>
+      </c>
+      <c r="BK21" t="inlineStr">
+        <is>
+          <t>$5.97</t>
+        </is>
+      </c>
+      <c r="BL21" t="inlineStr">
+        <is>
+          <t>That's Smart! Large Shell Eggs</t>
+        </is>
+      </c>
+      <c r="BM21" t="inlineStr">
+        <is>
+          <t>$5.97</t>
+        </is>
+      </c>
+      <c r="BN21" t="inlineStr">
+        <is>
+          <t>That's Smart! Large Shell Eggs</t>
+        </is>
+      </c>
+      <c r="BO21" t="inlineStr">
+        <is>
+          <t>$5.97</t>
+        </is>
+      </c>
+      <c r="BP21" t="inlineStr">
+        <is>
+          <t>That's Smart! Large Shell Eggs</t>
+        </is>
+      </c>
+      <c r="BQ21" t="inlineStr">
+        <is>
+          <t>$5.97</t>
+        </is>
+      </c>
+      <c r="BR21" t="inlineStr">
+        <is>
+          <t>That's Smart! Large Shell Eggs</t>
+        </is>
+      </c>
+      <c r="BS21" t="inlineStr">
+        <is>
+          <t>$5.97</t>
+        </is>
+      </c>
+      <c r="BT21" t="inlineStr">
+        <is>
+          <t>That's Smart! Large Shell Eggs</t>
+        </is>
+      </c>
+      <c r="BU21" t="inlineStr">
+        <is>
+          <t>$5.97</t>
+        </is>
+      </c>
+      <c r="BV21" t="inlineStr">
+        <is>
+          <t>That's Smart! Large Shell Eggs</t>
+        </is>
+      </c>
+      <c r="BW21" t="inlineStr">
+        <is>
+          <t>$5.97</t>
+        </is>
+      </c>
+      <c r="BX21" t="inlineStr">
+        <is>
+          <t>That's Smart! Large Shell Eggs</t>
+        </is>
+      </c>
+      <c r="BY21" t="inlineStr">
+        <is>
+          <t>$5.97</t>
+        </is>
+      </c>
+      <c r="BZ21" t="inlineStr">
+        <is>
+          <t>That's Smart! Large Shell Eggs</t>
+        </is>
+      </c>
+      <c r="CA21" t="inlineStr">
+        <is>
+          <t>$5.97</t>
+        </is>
+      </c>
+      <c r="CB21" t="inlineStr">
+        <is>
+          <t>That's Smart! Large Shell Eggs</t>
+        </is>
+      </c>
+      <c r="CC21" t="inlineStr">
+        <is>
+          <t>$5.97</t>
+        </is>
+      </c>
+      <c r="CD21" t="inlineStr">
+        <is>
+          <t>That's Smart! Large Shell Eggs</t>
+        </is>
+      </c>
+      <c r="CE21" t="inlineStr">
+        <is>
+          <t>$5.97</t>
+        </is>
+      </c>
+      <c r="CF21" t="inlineStr">
+        <is>
+          <t>That's Smart! Large Shell Eggs</t>
+        </is>
+      </c>
+      <c r="CG21" t="inlineStr">
+        <is>
+          <t>$5.97</t>
+        </is>
+      </c>
+      <c r="CH21" t="inlineStr">
+        <is>
+          <t>That's Smart! Large Shell Eggs</t>
+        </is>
+      </c>
+      <c r="CI21" t="inlineStr">
+        <is>
+          <t>$4.97</t>
+        </is>
+      </c>
+      <c r="CJ21" t="inlineStr">
+        <is>
+          <t>That's Smart! Large Shell Eggs</t>
+        </is>
+      </c>
+      <c r="CK21" t="inlineStr">
+        <is>
+          <t>$4.97</t>
+        </is>
+      </c>
+      <c r="CL21" t="inlineStr">
+        <is>
+          <t>That's Smart! Large Shell Eggs</t>
+        </is>
+      </c>
+      <c r="CM21" t="inlineStr">
+        <is>
+          <t>$4.97</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -6545,6 +9979,176 @@
           <t>748</t>
         </is>
       </c>
+      <c r="BF22" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="BG22" t="inlineStr">
+        <is>
+          <t>748</t>
+        </is>
+      </c>
+      <c r="BH22" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="BI22" t="inlineStr">
+        <is>
+          <t>748</t>
+        </is>
+      </c>
+      <c r="BJ22" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="BK22" t="inlineStr">
+        <is>
+          <t>748</t>
+        </is>
+      </c>
+      <c r="BL22" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="BM22" t="inlineStr">
+        <is>
+          <t>748</t>
+        </is>
+      </c>
+      <c r="BN22" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="BO22" t="inlineStr">
+        <is>
+          <t>748</t>
+        </is>
+      </c>
+      <c r="BP22" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="BQ22" t="inlineStr">
+        <is>
+          <t>748</t>
+        </is>
+      </c>
+      <c r="BR22" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="BS22" t="inlineStr">
+        <is>
+          <t>748</t>
+        </is>
+      </c>
+      <c r="BT22" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="BU22" t="inlineStr">
+        <is>
+          <t>748</t>
+        </is>
+      </c>
+      <c r="BV22" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="BW22" t="inlineStr">
+        <is>
+          <t>748</t>
+        </is>
+      </c>
+      <c r="BX22" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="BY22" t="inlineStr">
+        <is>
+          <t>748</t>
+        </is>
+      </c>
+      <c r="BZ22" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="CA22" t="inlineStr">
+        <is>
+          <t>748</t>
+        </is>
+      </c>
+      <c r="CB22" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="CC22" t="inlineStr">
+        <is>
+          <t>748</t>
+        </is>
+      </c>
+      <c r="CD22" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="CE22" t="inlineStr">
+        <is>
+          <t>748</t>
+        </is>
+      </c>
+      <c r="CF22" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="CG22" t="inlineStr">
+        <is>
+          <t>748</t>
+        </is>
+      </c>
+      <c r="CH22" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="CI22" t="inlineStr">
+        <is>
+          <t>748</t>
+        </is>
+      </c>
+      <c r="CJ22" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="CK22" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="CL22" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="CM22" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -6830,6 +10434,176 @@
       <c r="BE23" t="inlineStr">
         <is>
           <t>748</t>
+        </is>
+      </c>
+      <c r="BF23" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="BG23" t="inlineStr">
+        <is>
+          <t>748</t>
+        </is>
+      </c>
+      <c r="BH23" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="BI23" t="inlineStr">
+        <is>
+          <t>748</t>
+        </is>
+      </c>
+      <c r="BJ23" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="BK23" t="inlineStr">
+        <is>
+          <t>748</t>
+        </is>
+      </c>
+      <c r="BL23" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="BM23" t="inlineStr">
+        <is>
+          <t>748</t>
+        </is>
+      </c>
+      <c r="BN23" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="BO23" t="inlineStr">
+        <is>
+          <t>748</t>
+        </is>
+      </c>
+      <c r="BP23" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="BQ23" t="inlineStr">
+        <is>
+          <t>748</t>
+        </is>
+      </c>
+      <c r="BR23" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="BS23" t="inlineStr">
+        <is>
+          <t>748</t>
+        </is>
+      </c>
+      <c r="BT23" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="BU23" t="inlineStr">
+        <is>
+          <t>748</t>
+        </is>
+      </c>
+      <c r="BV23" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="BW23" t="inlineStr">
+        <is>
+          <t>748</t>
+        </is>
+      </c>
+      <c r="BX23" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="BY23" t="inlineStr">
+        <is>
+          <t>748</t>
+        </is>
+      </c>
+      <c r="BZ23" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="CA23" t="inlineStr">
+        <is>
+          <t>748</t>
+        </is>
+      </c>
+      <c r="CB23" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="CC23" t="inlineStr">
+        <is>
+          <t>748</t>
+        </is>
+      </c>
+      <c r="CD23" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="CE23" t="inlineStr">
+        <is>
+          <t>748</t>
+        </is>
+      </c>
+      <c r="CF23" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="CG23" t="inlineStr">
+        <is>
+          <t>748</t>
+        </is>
+      </c>
+      <c r="CH23" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="CI23" t="inlineStr">
+        <is>
+          <t>748</t>
+        </is>
+      </c>
+      <c r="CJ23" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="CK23" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="CL23" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="CM23" t="inlineStr">
+        <is>
+          <t>Not found</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Removed Icon file and updated spreadsheet
</commit_message>
<xml_diff>
--- a/price_extractor.xlsx
+++ b/price_extractor.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:FC23"/>
+  <dimension ref="A1:FG23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1224,6 +1224,26 @@
           <t>Price_2025-04-23 03:05</t>
         </is>
       </c>
+      <c r="FD1" s="1" t="inlineStr">
+        <is>
+          <t>Product Name_2025-04-24 03:04</t>
+        </is>
+      </c>
+      <c r="FE1" s="1" t="inlineStr">
+        <is>
+          <t>Price_2025-04-24 03:04</t>
+        </is>
+      </c>
+      <c r="FF1" s="1" t="inlineStr">
+        <is>
+          <t>Product Name_2025-04-25 03:05</t>
+        </is>
+      </c>
+      <c r="FG1" s="1" t="inlineStr">
+        <is>
+          <t>Price_2025-04-25 03:05</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -2021,6 +2041,26 @@
           <t>2.999</t>
         </is>
       </c>
+      <c r="FD2" t="inlineStr">
+        <is>
+          <t>UNLEADED 87 (10% ETH)</t>
+        </is>
+      </c>
+      <c r="FE2" t="inlineStr">
+        <is>
+          <t>2.999</t>
+        </is>
+      </c>
+      <c r="FF2" t="inlineStr">
+        <is>
+          <t>UNLEADED 87 (10% ETH)</t>
+        </is>
+      </c>
+      <c r="FG2" t="inlineStr">
+        <is>
+          <t>2.999</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -2818,6 +2858,26 @@
           <t>$2.87</t>
         </is>
       </c>
+      <c r="FD3" t="inlineStr">
+        <is>
+          <t>That's Smart! Fat Free Skim Milk</t>
+        </is>
+      </c>
+      <c r="FE3" t="inlineStr">
+        <is>
+          <t>$2.87</t>
+        </is>
+      </c>
+      <c r="FF3" t="inlineStr">
+        <is>
+          <t>That's Smart! Fat Free Skim Milk</t>
+        </is>
+      </c>
+      <c r="FG3" t="inlineStr">
+        <is>
+          <t>$2.87</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -3615,6 +3675,26 @@
           <t>32¢ ea.</t>
         </is>
       </c>
+      <c r="FD4" t="inlineStr">
+        <is>
+          <t>Roma Tomatoes</t>
+        </is>
+      </c>
+      <c r="FE4" t="inlineStr">
+        <is>
+          <t>32¢ ea.</t>
+        </is>
+      </c>
+      <c r="FF4" t="inlineStr">
+        <is>
+          <t>Roma Tomatoes</t>
+        </is>
+      </c>
+      <c r="FG4" t="inlineStr">
+        <is>
+          <t>32¢ ea.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -4412,6 +4492,26 @@
           <t>$4.59</t>
         </is>
       </c>
+      <c r="FD5" t="inlineStr">
+        <is>
+          <t>Quaker Cap'n Crunch Regular Cereal</t>
+        </is>
+      </c>
+      <c r="FE5" t="inlineStr">
+        <is>
+          <t>$4.59</t>
+        </is>
+      </c>
+      <c r="FF5" t="inlineStr">
+        <is>
+          <t>Quaker Cap'n Crunch Regular Cereal</t>
+        </is>
+      </c>
+      <c r="FG5" t="inlineStr">
+        <is>
+          <t>$4.59</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -5209,6 +5309,26 @@
           <t>$3.99</t>
         </is>
       </c>
+      <c r="FD6" t="inlineStr">
+        <is>
+          <t>Sara Lee Artesano Brioche Buns, 8 count</t>
+        </is>
+      </c>
+      <c r="FE6" t="inlineStr">
+        <is>
+          <t>$3.99</t>
+        </is>
+      </c>
+      <c r="FF6" t="inlineStr">
+        <is>
+          <t>Sara Lee Artesano Brioche Buns, 8 count</t>
+        </is>
+      </c>
+      <c r="FG6" t="inlineStr">
+        <is>
+          <t>$3.99</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -6006,6 +6126,26 @@
           <t>$3.65</t>
         </is>
       </c>
+      <c r="FD7" t="inlineStr">
+        <is>
+          <t>That's Smart! Mayonnaise</t>
+        </is>
+      </c>
+      <c r="FE7" t="inlineStr">
+        <is>
+          <t>$3.65</t>
+        </is>
+      </c>
+      <c r="FF7" t="inlineStr">
+        <is>
+          <t>That's Smart! Mayonnaise</t>
+        </is>
+      </c>
+      <c r="FG7" t="inlineStr">
+        <is>
+          <t>$3.65</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -6803,6 +6943,26 @@
           <t>$1.99</t>
         </is>
       </c>
+      <c r="FD8" t="inlineStr">
+        <is>
+          <t>Hy-Vee Light Bartlett Pear Halves In Pear Juice From Concentrate</t>
+        </is>
+      </c>
+      <c r="FE8" t="inlineStr">
+        <is>
+          <t>$1.99</t>
+        </is>
+      </c>
+      <c r="FF8" t="inlineStr">
+        <is>
+          <t>Hy-Vee Light Bartlett Pear Halves In Pear Juice From Concentrate</t>
+        </is>
+      </c>
+      <c r="FG8" t="inlineStr">
+        <is>
+          <t>$1.99</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -7600,6 +7760,26 @@
           <t>$3.99</t>
         </is>
       </c>
+      <c r="FD9" t="inlineStr">
+        <is>
+          <t>Dole Fresh Romaine Hearts</t>
+        </is>
+      </c>
+      <c r="FE9" t="inlineStr">
+        <is>
+          <t>$3.99</t>
+        </is>
+      </c>
+      <c r="FF9" t="inlineStr">
+        <is>
+          <t>Dole Fresh Romaine Hearts</t>
+        </is>
+      </c>
+      <c r="FG9" t="inlineStr">
+        <is>
+          <t>$3.99</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -8397,6 +8577,26 @@
           <t>$5.79</t>
         </is>
       </c>
+      <c r="FD10" t="inlineStr">
+        <is>
+          <t>Hy-Vee Oven Roasted Cured Turkey Breast &amp; White Turkey Shaved Slices</t>
+        </is>
+      </c>
+      <c r="FE10" t="inlineStr">
+        <is>
+          <t>$5.79</t>
+        </is>
+      </c>
+      <c r="FF10" t="inlineStr">
+        <is>
+          <t>Hy-Vee Oven Roasted Cured Turkey Breast &amp; White Turkey Shaved Slices</t>
+        </is>
+      </c>
+      <c r="FG10" t="inlineStr">
+        <is>
+          <t>$5.79</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -9194,6 +9394,26 @@
           <t>$3.29</t>
         </is>
       </c>
+      <c r="FD11" t="inlineStr">
+        <is>
+          <t>That's Smart! Small Curd Cottage Cheese 4% Milkfat</t>
+        </is>
+      </c>
+      <c r="FE11" t="inlineStr">
+        <is>
+          <t>$3.29</t>
+        </is>
+      </c>
+      <c r="FF11" t="inlineStr">
+        <is>
+          <t>That's Smart! Small Curd Cottage Cheese 4% Milkfat</t>
+        </is>
+      </c>
+      <c r="FG11" t="inlineStr">
+        <is>
+          <t>$3.29</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -9991,6 +10211,26 @@
           <t>$4.97</t>
         </is>
       </c>
+      <c r="FD12" t="inlineStr">
+        <is>
+          <t>Fairlife Fat Free Ultra-Filtered Milk</t>
+        </is>
+      </c>
+      <c r="FE12" t="inlineStr">
+        <is>
+          <t>$4.97</t>
+        </is>
+      </c>
+      <c r="FF12" t="inlineStr">
+        <is>
+          <t>Fairlife Fat Free Ultra-Filtered Milk</t>
+        </is>
+      </c>
+      <c r="FG12" t="inlineStr">
+        <is>
+          <t>$4.97</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -10788,6 +11028,26 @@
           <t>Not found</t>
         </is>
       </c>
+      <c r="FD13" t="inlineStr">
+        <is>
+          <t>Fresh Chiquita Bananas</t>
+        </is>
+      </c>
+      <c r="FE13" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="FF13" t="inlineStr">
+        <is>
+          <t>Fresh Chiquita Bananas</t>
+        </is>
+      </c>
+      <c r="FG13" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -11585,6 +11845,26 @@
           <t>$5.99</t>
         </is>
       </c>
+      <c r="FD14" t="inlineStr">
+        <is>
+          <t>Wonderful Halos Mandarin Oranges</t>
+        </is>
+      </c>
+      <c r="FE14" t="inlineStr">
+        <is>
+          <t>$5.99</t>
+        </is>
+      </c>
+      <c r="FF14" t="inlineStr">
+        <is>
+          <t>Wonderful Halos Mandarin Oranges</t>
+        </is>
+      </c>
+      <c r="FG14" t="inlineStr">
+        <is>
+          <t>$5.99</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -12382,6 +12662,26 @@
           <t>$7.49/lb</t>
         </is>
       </c>
+      <c r="FD15" t="inlineStr">
+        <is>
+          <t>Certified Ground Round 90% Lean 10% Fat</t>
+        </is>
+      </c>
+      <c r="FE15" t="inlineStr">
+        <is>
+          <t>$7.49/lb</t>
+        </is>
+      </c>
+      <c r="FF15" t="inlineStr">
+        <is>
+          <t>Certified Ground Round 90% Lean 10% Fat</t>
+        </is>
+      </c>
+      <c r="FG15" t="inlineStr">
+        <is>
+          <t>$7.49/lb</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -13179,6 +13479,26 @@
           <t>$4.34 ea.</t>
         </is>
       </c>
+      <c r="FD16" t="inlineStr">
+        <is>
+          <t>Boneless Skinless Chicken Breast</t>
+        </is>
+      </c>
+      <c r="FE16" t="inlineStr">
+        <is>
+          <t>$4.34 ea.</t>
+        </is>
+      </c>
+      <c r="FF16" t="inlineStr">
+        <is>
+          <t>Boneless Skinless Chicken Breast</t>
+        </is>
+      </c>
+      <c r="FG16" t="inlineStr">
+        <is>
+          <t>$4.34 ea.</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -13976,6 +14296,26 @@
           <t>$40,275</t>
         </is>
       </c>
+      <c r="FD17" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="FE17" t="inlineStr">
+        <is>
+          <t>$40,275</t>
+        </is>
+      </c>
+      <c r="FF17" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="FG17" t="inlineStr">
+        <is>
+          <t>$40,275</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -14589,6 +14929,26 @@
         </is>
       </c>
       <c r="FC18" t="inlineStr">
+        <is>
+          <t>$37,000*</t>
+        </is>
+      </c>
+      <c r="FD18" t="inlineStr">
+        <is>
+          <t>Silverado</t>
+        </is>
+      </c>
+      <c r="FE18" t="inlineStr">
+        <is>
+          <t>$37,000*</t>
+        </is>
+      </c>
+      <c r="FF18" t="inlineStr">
+        <is>
+          <t>Silverado</t>
+        </is>
+      </c>
+      <c r="FG18" t="inlineStr">
         <is>
           <t>$37,000*</t>
         </is>
@@ -15238,6 +15598,26 @@
           <t>$3.94</t>
         </is>
       </c>
+      <c r="FD19" t="inlineStr">
+        <is>
+          <t>2 x 4 x 8' Construction/Framing Lumber</t>
+        </is>
+      </c>
+      <c r="FE19" t="inlineStr">
+        <is>
+          <t>$3.94</t>
+        </is>
+      </c>
+      <c r="FF19" t="inlineStr">
+        <is>
+          <t>2 x 4 x 8' Construction/Framing Lumber</t>
+        </is>
+      </c>
+      <c r="FG19" t="inlineStr">
+        <is>
+          <t>$3.94</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -16035,6 +16415,26 @@
           <t>$6.99</t>
         </is>
       </c>
+      <c r="FD20" t="inlineStr">
+        <is>
+          <t>Hy-Vee Select 100% Pure Maple Syrup</t>
+        </is>
+      </c>
+      <c r="FE20" t="inlineStr">
+        <is>
+          <t>$6.99</t>
+        </is>
+      </c>
+      <c r="FF20" t="inlineStr">
+        <is>
+          <t>Hy-Vee Select 100% Pure Maple Syrup</t>
+        </is>
+      </c>
+      <c r="FG20" t="inlineStr">
+        <is>
+          <t>$6.99</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -16832,6 +17232,26 @@
           <t>$4.47</t>
         </is>
       </c>
+      <c r="FD21" t="inlineStr">
+        <is>
+          <t>That's Smart! Large Shell Eggs</t>
+        </is>
+      </c>
+      <c r="FE21" t="inlineStr">
+        <is>
+          <t>$4.47</t>
+        </is>
+      </c>
+      <c r="FF21" t="inlineStr">
+        <is>
+          <t>That's Smart! Large Shell Eggs</t>
+        </is>
+      </c>
+      <c r="FG21" t="inlineStr">
+        <is>
+          <t>$4.47</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -17517,6 +17937,18 @@
         </is>
       </c>
       <c r="FC22" t="inlineStr"/>
+      <c r="FD22" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="FE22" t="inlineStr"/>
+      <c r="FF22" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="FG22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -18202,6 +18634,18 @@
         </is>
       </c>
       <c r="FC23" t="inlineStr"/>
+      <c r="FD23" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="FE23" t="inlineStr"/>
+      <c r="FF23" t="inlineStr">
+        <is>
+          <t>Not found</t>
+        </is>
+      </c>
+      <c r="FG23" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>